<commit_message>
docs: use HijrahDate in spec; mark EN plural rows in copy deck
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/copy/izzah-copy-id-en.xlsx
+++ b/docs/copy/izzah-copy-id-en.xlsx
@@ -3430,7 +3430,7 @@
       </c>
       <c r="F82" s="5" t="inlineStr">
         <is>
-          <t>day / days</t>
+          <t>days</t>
         </is>
       </c>
       <c r="G82" s="5" t="inlineStr">
@@ -4362,7 +4362,7 @@
       </c>
       <c r="G109" s="5" t="inlineStr">
         <is>
-          <t>Rendered UPPERCASE, countdown 60→0.</t>
+          <t>Rendered UPPERCASE, countdown 60→0. PLURAL in EN.</t>
         </is>
       </c>
       <c r="H109" s="6" t="inlineStr"/>
@@ -8058,7 +8058,11 @@
           <t>{n} days</t>
         </is>
       </c>
-      <c r="G219" s="5" t="inlineStr"/>
+      <c r="G219" s="5" t="inlineStr">
+        <is>
+          <t>PLURAL in EN.</t>
+        </is>
+      </c>
       <c r="H219" s="6" t="inlineStr"/>
       <c r="I219" s="6" t="inlineStr"/>
     </row>
@@ -9280,7 +9284,7 @@
       </c>
       <c r="G255" s="7" t="inlineStr">
         <is>
-          <t>After 5 wrong PINs: 30 s cooldown.</t>
+          <t>After 5 wrong PINs: 30 s cooldown. PLURAL in EN.</t>
         </is>
       </c>
       <c r="H255" s="6" t="inlineStr"/>

</xml_diff>

<commit_message>
feat(protect): schedules, app picker and shield UI
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/copy/izzah-copy-id-en.xlsx
+++ b/docs/copy/izzah-copy-id-en.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Glossary" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Copy'!$A$1:$I$280</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Copy'!$A$1:$I$291</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Religious'!$A$1:$I$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Glossary'!$A$1:$E$13</definedName>
   </definedNames>
@@ -631,7 +631,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I280"/>
+  <dimension ref="A1:I291"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -7342,74 +7342,74 @@
       <c r="I198" s="6" t="inlineStr"/>
     </row>
     <row r="199">
-      <c r="A199" s="5" t="n">
+      <c r="A199" s="7" t="n">
         <v>198</v>
       </c>
-      <c r="B199" s="5" t="inlineStr">
-        <is>
-          <t>shield_label</t>
-        </is>
-      </c>
-      <c r="C199" s="5" t="inlineStr">
-        <is>
-          <t>Layar terkunci</t>
-        </is>
-      </c>
-      <c r="D199" s="5" t="inlineStr">
-        <is>
-          <t>DESIGN</t>
-        </is>
-      </c>
-      <c r="E199" s="5" t="inlineStr">
-        <is>
-          <t>Waktu terjaga · sampai {time}</t>
-        </is>
-      </c>
-      <c r="F199" s="5" t="inlineStr">
-        <is>
-          <t>Guarded hours · until {time}</t>
-        </is>
-      </c>
-      <c r="G199" s="5" t="inlineStr">
-        <is>
-          <t>Rendered UPPERCASE.</t>
+      <c r="B199" s="7" t="inlineStr">
+        <is>
+          <t>keeprun_title</t>
+        </is>
+      </c>
+      <c r="C199" s="7" t="inlineStr">
+        <is>
+          <t>Lindungi</t>
+        </is>
+      </c>
+      <c r="D199" s="7" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="E199" s="7" t="inlineStr">
+        <is>
+          <t>Biarkan Izzah tetap berjalan</t>
+        </is>
+      </c>
+      <c r="F199" s="7" t="inlineStr">
+        <is>
+          <t>Keep Izzah running</t>
+        </is>
+      </c>
+      <c r="G199" s="7" t="inlineStr">
+        <is>
+          <t>Xiaomi/Redmi/POCO only. Written for the Android build, needs review.</t>
         </is>
       </c>
       <c r="H199" s="6" t="inlineStr"/>
       <c r="I199" s="6" t="inlineStr"/>
     </row>
     <row r="200">
-      <c r="A200" s="5" t="n">
+      <c r="A200" s="7" t="n">
         <v>199</v>
       </c>
-      <c r="B200" s="5" t="inlineStr">
-        <is>
-          <t>shield_title</t>
-        </is>
-      </c>
-      <c r="C200" s="5" t="inlineStr">
-        <is>
-          <t>Layar terkunci</t>
-        </is>
-      </c>
-      <c r="D200" s="5" t="inlineStr">
-        <is>
-          <t>DESIGN</t>
-        </is>
-      </c>
-      <c r="E200" s="5" t="inlineStr">
-        <is>
-          <t>Sudah larut. Istirahat dulu, yuk.</t>
-        </is>
-      </c>
-      <c r="F200" s="5" t="inlineStr">
-        <is>
-          <t>It's late. Time to rest, okay?</t>
-        </is>
-      </c>
-      <c r="G200" s="5" t="inlineStr">
-        <is>
-          <t>Fits a late-night slot only. A daytime variant is proposed below.</t>
+      <c r="B200" s="7" t="inlineStr">
+        <is>
+          <t>keeprun_desc</t>
+        </is>
+      </c>
+      <c r="C200" s="7" t="inlineStr">
+        <is>
+          <t>Lindungi</t>
+        </is>
+      </c>
+      <c r="D200" s="7" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="E200" s="7" t="inlineStr">
+        <is>
+          <t>HP-mu bisa menghentikan Izzah di latar belakang. Izinkan Autostart dan lepas batas baterai supaya pagar tetap berfungsi.</t>
+        </is>
+      </c>
+      <c r="F200" s="7" t="inlineStr">
+        <is>
+          <t>Your phone may stop Izzah in the background. Allow Autostart and remove the battery limit so the fence keeps working.</t>
+        </is>
+      </c>
+      <c r="G200" s="7" t="inlineStr">
+        <is>
+          <t>Needs review.</t>
         </is>
       </c>
       <c r="H200" s="6" t="inlineStr"/>
@@ -7421,12 +7421,12 @@
       </c>
       <c r="B201" s="7" t="inlineStr">
         <is>
-          <t>shield_title_day</t>
+          <t>keeprun_autostart</t>
         </is>
       </c>
       <c r="C201" s="7" t="inlineStr">
         <is>
-          <t>Layar terkunci</t>
+          <t>Lindungi</t>
         </is>
       </c>
       <c r="D201" s="7" t="inlineStr">
@@ -7436,118 +7436,130 @@
       </c>
       <c r="E201" s="7" t="inlineStr">
         <is>
-          <t>Sebentar dulu. Tarik napas, yuk.</t>
+          <t>Izinkan Autostart</t>
         </is>
       </c>
       <c r="F201" s="7" t="inlineStr">
         <is>
-          <t>Hold on a moment. Let's take a breath.</t>
+          <t>Allow Autostart</t>
         </is>
       </c>
       <c r="G201" s="7" t="inlineStr">
         <is>
-          <t>For daytime slots (e.g. 13.00–15.00).</t>
+          <t>Opens the vendor Autostart screen.</t>
         </is>
       </c>
       <c r="H201" s="6" t="inlineStr"/>
       <c r="I201" s="6" t="inlineStr"/>
     </row>
     <row r="202">
-      <c r="A202" s="5" t="n">
+      <c r="A202" s="7" t="n">
         <v>201</v>
       </c>
-      <c r="B202" s="5" t="inlineStr">
-        <is>
-          <t>shield_body</t>
-        </is>
-      </c>
-      <c r="C202" s="5" t="inlineStr">
-        <is>
-          <t>Layar terkunci</t>
-        </is>
-      </c>
-      <c r="D202" s="5" t="inlineStr">
-        <is>
-          <t>DESIGN</t>
-        </is>
-      </c>
-      <c r="E202" s="5" t="inlineStr">
-        <is>
-          <t>Kamu sendiri yang memasang pagar ini, di saat kamu sedang kuat.</t>
-        </is>
-      </c>
-      <c r="F202" s="5" t="inlineStr">
-        <is>
-          <t>You put up this fence yourself, at a moment you were strong.</t>
-        </is>
-      </c>
-      <c r="G202" s="5" t="inlineStr"/>
+      <c r="B202" s="7" t="inlineStr">
+        <is>
+          <t>keeprun_battery</t>
+        </is>
+      </c>
+      <c r="C202" s="7" t="inlineStr">
+        <is>
+          <t>Lindungi</t>
+        </is>
+      </c>
+      <c r="D202" s="7" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="E202" s="7" t="inlineStr">
+        <is>
+          <t>Lepas batas baterai</t>
+        </is>
+      </c>
+      <c r="F202" s="7" t="inlineStr">
+        <is>
+          <t>Remove battery limit</t>
+        </is>
+      </c>
+      <c r="G202" s="7" t="inlineStr">
+        <is>
+          <t>Opens the vendor battery screen.</t>
+        </is>
+      </c>
       <c r="H202" s="6" t="inlineStr"/>
       <c r="I202" s="6" t="inlineStr"/>
     </row>
     <row r="203">
-      <c r="A203" s="5" t="n">
+      <c r="A203" s="7" t="n">
         <v>202</v>
       </c>
-      <c r="B203" s="5" t="inlineStr">
-        <is>
-          <t>shield_take_jeda</t>
-        </is>
-      </c>
-      <c r="C203" s="5" t="inlineStr">
-        <is>
-          <t>Layar terkunci</t>
-        </is>
-      </c>
-      <c r="D203" s="5" t="inlineStr">
-        <is>
-          <t>DESIGN</t>
-        </is>
-      </c>
-      <c r="E203" s="5" t="inlineStr">
-        <is>
-          <t>Ambil jeda 60 detik</t>
-        </is>
-      </c>
-      <c r="F203" s="5" t="inlineStr">
-        <is>
-          <t>Take a 60-second pause</t>
-        </is>
-      </c>
-      <c r="G203" s="5" t="inlineStr"/>
+      <c r="B203" s="7" t="inlineStr">
+        <is>
+          <t>keeprun_done</t>
+        </is>
+      </c>
+      <c r="C203" s="7" t="inlineStr">
+        <is>
+          <t>Lindungi</t>
+        </is>
+      </c>
+      <c r="D203" s="7" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="E203" s="7" t="inlineStr">
+        <is>
+          <t>Sudah kuatur</t>
+        </is>
+      </c>
+      <c r="F203" s="7" t="inlineStr">
+        <is>
+          <t>All set</t>
+        </is>
+      </c>
+      <c r="G203" s="7" t="inlineStr">
+        <is>
+          <t>Hides the card for good.</t>
+        </is>
+      </c>
       <c r="H203" s="6" t="inlineStr"/>
       <c r="I203" s="6" t="inlineStr"/>
     </row>
     <row r="204">
-      <c r="A204" s="5" t="n">
+      <c r="A204" s="7" t="n">
         <v>203</v>
       </c>
-      <c r="B204" s="5" t="inlineStr">
-        <is>
-          <t>shield_close_app</t>
-        </is>
-      </c>
-      <c r="C204" s="5" t="inlineStr">
-        <is>
-          <t>Layar terkunci</t>
-        </is>
-      </c>
-      <c r="D204" s="5" t="inlineStr">
-        <is>
-          <t>DESIGN</t>
-        </is>
-      </c>
-      <c r="E204" s="5" t="inlineStr">
-        <is>
-          <t>Tutup aplikasi</t>
-        </is>
-      </c>
-      <c r="F204" s="5" t="inlineStr">
-        <is>
-          <t>Close the app</t>
-        </is>
-      </c>
-      <c r="G204" s="5" t="inlineStr"/>
+      <c r="B204" s="7" t="inlineStr">
+        <is>
+          <t>apppicker_title</t>
+        </is>
+      </c>
+      <c r="C204" s="7" t="inlineStr">
+        <is>
+          <t>Pilih aplikasi</t>
+        </is>
+      </c>
+      <c r="D204" s="7" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="E204" s="7" t="inlineStr">
+        <is>
+          <t>Pilih aplikasi</t>
+        </is>
+      </c>
+      <c r="F204" s="7" t="inlineStr">
+        <is>
+          <t>Choose apps</t>
+        </is>
+      </c>
+      <c r="G204" s="7" t="inlineStr">
+        <is>
+          <t>Title of the app picker opened from Protect. Needs review.</t>
+        </is>
+      </c>
       <c r="H204" s="6" t="inlineStr"/>
       <c r="I204" s="6" t="inlineStr"/>
     </row>
@@ -7557,12 +7569,12 @@
       </c>
       <c r="B205" s="7" t="inlineStr">
         <is>
-          <t>shield_continue</t>
+          <t>apppicker_suggested</t>
         </is>
       </c>
       <c r="C205" s="7" t="inlineStr">
         <is>
-          <t>Layar terkunci</t>
+          <t>Pilih aplikasi</t>
         </is>
       </c>
       <c r="D205" s="7" t="inlineStr">
@@ -7572,151 +7584,167 @@
       </c>
       <c r="E205" s="7" t="inlineStr">
         <is>
-          <t>Tetap lanjutkan</t>
+          <t>Disarankan</t>
         </is>
       </c>
       <c r="F205" s="7" t="inlineStr">
         <is>
-          <t>Continue anyway</t>
+          <t>Suggested</t>
         </is>
       </c>
       <c r="G205" s="7" t="inlineStr">
         <is>
-          <t>Needed for 'Pengingat lembut' mode, where the design has no continue button.</t>
+          <t>Small header over the suggested browsers and social apps that are installed.</t>
         </is>
       </c>
       <c r="H205" s="6" t="inlineStr"/>
       <c r="I205" s="6" t="inlineStr"/>
     </row>
     <row r="206">
-      <c r="A206" s="5" t="n">
+      <c r="A206" s="7" t="n">
         <v>205</v>
       </c>
-      <c r="B206" s="5" t="inlineStr">
-        <is>
-          <t>shield_note_gentle</t>
-        </is>
-      </c>
-      <c r="C206" s="5" t="inlineStr">
-        <is>
-          <t>Layar terkunci</t>
-        </is>
-      </c>
-      <c r="D206" s="5" t="inlineStr">
-        <is>
-          <t>DESIGN</t>
-        </is>
-      </c>
-      <c r="E206" s="5" t="inlineStr">
-        <is>
-          <t>Kamu tetap bisa melanjutkan jika memang perlu</t>
-        </is>
-      </c>
-      <c r="F206" s="5" t="inlineStr">
-        <is>
-          <t>You can still continue if you really need to</t>
-        </is>
-      </c>
-      <c r="G206" s="5" t="inlineStr"/>
+      <c r="B206" s="7" t="inlineStr">
+        <is>
+          <t>apppicker_all</t>
+        </is>
+      </c>
+      <c r="C206" s="7" t="inlineStr">
+        <is>
+          <t>Pilih aplikasi</t>
+        </is>
+      </c>
+      <c r="D206" s="7" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="E206" s="7" t="inlineStr">
+        <is>
+          <t>Semua aplikasi</t>
+        </is>
+      </c>
+      <c r="F206" s="7" t="inlineStr">
+        <is>
+          <t>All apps</t>
+        </is>
+      </c>
+      <c r="G206" s="7" t="inlineStr">
+        <is>
+          <t>Small header over the alphabetical list.</t>
+        </is>
+      </c>
       <c r="H206" s="6" t="inlineStr"/>
       <c r="I206" s="6" t="inlineStr"/>
     </row>
     <row r="207">
-      <c r="A207" s="5" t="n">
+      <c r="A207" s="7" t="n">
         <v>206</v>
       </c>
-      <c r="B207" s="5" t="inlineStr">
-        <is>
-          <t>shield_note_pause</t>
-        </is>
-      </c>
-      <c r="C207" s="5" t="inlineStr">
-        <is>
-          <t>Layar terkunci</t>
-        </is>
-      </c>
-      <c r="D207" s="5" t="inlineStr">
-        <is>
-          <t>DESIGN</t>
-        </is>
-      </c>
-      <c r="E207" s="5" t="inlineStr">
-        <is>
-          <t>Setelah jeda, aplikasi terbuka 5 menit</t>
-        </is>
-      </c>
-      <c r="F207" s="5" t="inlineStr">
-        <is>
-          <t>After the pause, the app opens for 5 minutes</t>
-        </is>
-      </c>
-      <c r="G207" s="5" t="inlineStr"/>
+      <c r="B207" s="7" t="inlineStr">
+        <is>
+          <t>apppicker_search</t>
+        </is>
+      </c>
+      <c r="C207" s="7" t="inlineStr">
+        <is>
+          <t>Pilih aplikasi</t>
+        </is>
+      </c>
+      <c r="D207" s="7" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="E207" s="7" t="inlineStr">
+        <is>
+          <t>Cari aplikasi</t>
+        </is>
+      </c>
+      <c r="F207" s="7" t="inlineStr">
+        <is>
+          <t>Search apps</t>
+        </is>
+      </c>
+      <c r="G207" s="7" t="inlineStr">
+        <is>
+          <t>Search field placeholder.</t>
+        </is>
+      </c>
       <c r="H207" s="6" t="inlineStr"/>
       <c r="I207" s="6" t="inlineStr"/>
     </row>
     <row r="208">
-      <c r="A208" s="5" t="n">
+      <c r="A208" s="7" t="n">
         <v>207</v>
       </c>
-      <c r="B208" s="5" t="inlineStr">
-        <is>
-          <t>shield_note_full</t>
-        </is>
-      </c>
-      <c r="C208" s="5" t="inlineStr">
-        <is>
-          <t>Layar terkunci</t>
-        </is>
-      </c>
-      <c r="D208" s="5" t="inlineStr">
-        <is>
-          <t>DESIGN</t>
-        </is>
-      </c>
-      <c r="E208" s="5" t="inlineStr">
-        <is>
-          <t>Terbuka lagi pukul {time}</t>
-        </is>
-      </c>
-      <c r="F208" s="5" t="inlineStr">
-        <is>
-          <t>Opens again at {time}</t>
-        </is>
-      </c>
-      <c r="G208" s="5" t="inlineStr"/>
+      <c r="B208" s="7" t="inlineStr">
+        <is>
+          <t>slot_edit_from</t>
+        </is>
+      </c>
+      <c r="C208" s="7" t="inlineStr">
+        <is>
+          <t>Lindungi</t>
+        </is>
+      </c>
+      <c r="D208" s="7" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="E208" s="7" t="inlineStr">
+        <is>
+          <t>Dari</t>
+        </is>
+      </c>
+      <c r="F208" s="7" t="inlineStr">
+        <is>
+          <t>From</t>
+        </is>
+      </c>
+      <c r="G208" s="7" t="inlineStr">
+        <is>
+          <t>Label above the start time picker in the schedule editor. Needs review.</t>
+        </is>
+      </c>
       <c r="H208" s="6" t="inlineStr"/>
       <c r="I208" s="6" t="inlineStr"/>
     </row>
     <row r="209">
-      <c r="A209" s="5" t="n">
+      <c r="A209" s="7" t="n">
         <v>208</v>
       </c>
-      <c r="B209" s="5" t="inlineStr">
-        <is>
-          <t>settings_title</t>
-        </is>
-      </c>
-      <c r="C209" s="5" t="inlineStr">
-        <is>
-          <t>Pengaturan</t>
-        </is>
-      </c>
-      <c r="D209" s="5" t="inlineStr">
-        <is>
-          <t>DESIGN</t>
-        </is>
-      </c>
-      <c r="E209" s="5" t="inlineStr">
-        <is>
-          <t>Pengaturan</t>
-        </is>
-      </c>
-      <c r="F209" s="5" t="inlineStr">
-        <is>
-          <t>Settings</t>
-        </is>
-      </c>
-      <c r="G209" s="5" t="inlineStr"/>
+      <c r="B209" s="7" t="inlineStr">
+        <is>
+          <t>slot_edit_to</t>
+        </is>
+      </c>
+      <c r="C209" s="7" t="inlineStr">
+        <is>
+          <t>Lindungi</t>
+        </is>
+      </c>
+      <c r="D209" s="7" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="E209" s="7" t="inlineStr">
+        <is>
+          <t>Sampai</t>
+        </is>
+      </c>
+      <c r="F209" s="7" t="inlineStr">
+        <is>
+          <t>To</t>
+        </is>
+      </c>
+      <c r="G209" s="7" t="inlineStr">
+        <is>
+          <t>Label above the end time picker in the schedule editor. Needs review.</t>
+        </is>
+      </c>
       <c r="H209" s="6" t="inlineStr"/>
       <c r="I209" s="6" t="inlineStr"/>
     </row>
@@ -7726,12 +7754,12 @@
       </c>
       <c r="B210" s="5" t="inlineStr">
         <is>
-          <t>settings_profile_title</t>
+          <t>shield_label</t>
         </is>
       </c>
       <c r="C210" s="5" t="inlineStr">
         <is>
-          <t>Pengaturan</t>
+          <t>Layar terkunci</t>
         </is>
       </c>
       <c r="D210" s="5" t="inlineStr">
@@ -7741,15 +7769,19 @@
       </c>
       <c r="E210" s="5" t="inlineStr">
         <is>
-          <t>Akun anonim</t>
+          <t>Waktu terjaga · sampai {time}</t>
         </is>
       </c>
       <c r="F210" s="5" t="inlineStr">
         <is>
-          <t>Anonymous account</t>
-        </is>
-      </c>
-      <c r="G210" s="5" t="inlineStr"/>
+          <t>Guarded hours · until {time}</t>
+        </is>
+      </c>
+      <c r="G210" s="5" t="inlineStr">
+        <is>
+          <t>Rendered UPPERCASE.</t>
+        </is>
+      </c>
       <c r="H210" s="6" t="inlineStr"/>
       <c r="I210" s="6" t="inlineStr"/>
     </row>
@@ -7759,12 +7791,12 @@
       </c>
       <c r="B211" s="5" t="inlineStr">
         <is>
-          <t>settings_profile_sub</t>
+          <t>shield_title</t>
         </is>
       </c>
       <c r="C211" s="5" t="inlineStr">
         <is>
-          <t>Pengaturan</t>
+          <t>Layar terkunci</t>
         </is>
       </c>
       <c r="D211" s="5" t="inlineStr">
@@ -7774,85 +7806,89 @@
       </c>
       <c r="E211" s="5" t="inlineStr">
         <is>
-          <t>Tanpa email · data hanya di HP ini</t>
+          <t>Sudah larut. Istirahat dulu, yuk.</t>
         </is>
       </c>
       <c r="F211" s="5" t="inlineStr">
         <is>
-          <t>No email · data stays on this phone</t>
-        </is>
-      </c>
-      <c r="G211" s="5" t="inlineStr"/>
+          <t>It's late. Time to rest, okay?</t>
+        </is>
+      </c>
+      <c r="G211" s="5" t="inlineStr">
+        <is>
+          <t>Fits a late-night slot only. A daytime variant is proposed below.</t>
+        </is>
+      </c>
       <c r="H211" s="6" t="inlineStr"/>
       <c r="I211" s="6" t="inlineStr"/>
     </row>
     <row r="212">
-      <c r="A212" s="5" t="n">
+      <c r="A212" s="7" t="n">
         <v>211</v>
       </c>
-      <c r="B212" s="5" t="inlineStr">
-        <is>
-          <t>settings_group_privacy</t>
-        </is>
-      </c>
-      <c r="C212" s="5" t="inlineStr">
-        <is>
-          <t>Pengaturan</t>
-        </is>
-      </c>
-      <c r="D212" s="5" t="inlineStr">
-        <is>
-          <t>DESIGN</t>
-        </is>
-      </c>
-      <c r="E212" s="5" t="inlineStr">
-        <is>
-          <t>Privasi</t>
-        </is>
-      </c>
-      <c r="F212" s="5" t="inlineStr">
-        <is>
-          <t>Privacy</t>
-        </is>
-      </c>
-      <c r="G212" s="5" t="inlineStr"/>
+      <c r="B212" s="7" t="inlineStr">
+        <is>
+          <t>shield_title_day</t>
+        </is>
+      </c>
+      <c r="C212" s="7" t="inlineStr">
+        <is>
+          <t>Layar terkunci</t>
+        </is>
+      </c>
+      <c r="D212" s="7" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="E212" s="7" t="inlineStr">
+        <is>
+          <t>Sebentar dulu. Tarik napas, yuk.</t>
+        </is>
+      </c>
+      <c r="F212" s="7" t="inlineStr">
+        <is>
+          <t>Hold on a moment. Let's take a breath.</t>
+        </is>
+      </c>
+      <c r="G212" s="7" t="inlineStr">
+        <is>
+          <t>For daytime slots (e.g. 13.00–15.00).</t>
+        </is>
+      </c>
       <c r="H212" s="6" t="inlineStr"/>
       <c r="I212" s="6" t="inlineStr"/>
     </row>
     <row r="213">
-      <c r="A213" s="8" t="n">
+      <c r="A213" s="5" t="n">
         <v>212</v>
       </c>
-      <c r="B213" s="8" t="inlineStr">
-        <is>
-          <t>settings_pin_lock</t>
-        </is>
-      </c>
-      <c r="C213" s="8" t="inlineStr">
-        <is>
-          <t>Pengaturan</t>
-        </is>
-      </c>
-      <c r="D213" s="8" t="inlineStr">
-        <is>
-          <t>ANDROID</t>
-        </is>
-      </c>
-      <c r="E213" s="8" t="inlineStr">
-        <is>
-          <t>Kunci dengan PIN &amp; sidik jari</t>
-        </is>
-      </c>
-      <c r="F213" s="8" t="inlineStr">
-        <is>
-          <t>Lock with PIN &amp; fingerprint</t>
-        </is>
-      </c>
-      <c r="G213" s="8" t="inlineStr">
-        <is>
-          <t>Original: '…&amp; Face ID'.</t>
-        </is>
-      </c>
+      <c r="B213" s="5" t="inlineStr">
+        <is>
+          <t>shield_body</t>
+        </is>
+      </c>
+      <c r="C213" s="5" t="inlineStr">
+        <is>
+          <t>Layar terkunci</t>
+        </is>
+      </c>
+      <c r="D213" s="5" t="inlineStr">
+        <is>
+          <t>DESIGN</t>
+        </is>
+      </c>
+      <c r="E213" s="5" t="inlineStr">
+        <is>
+          <t>Kamu sendiri yang memasang pagar ini, di saat kamu sedang kuat.</t>
+        </is>
+      </c>
+      <c r="F213" s="5" t="inlineStr">
+        <is>
+          <t>You put up this fence yourself, at a moment you were strong.</t>
+        </is>
+      </c>
+      <c r="G213" s="5" t="inlineStr"/>
       <c r="H213" s="6" t="inlineStr"/>
       <c r="I213" s="6" t="inlineStr"/>
     </row>
@@ -7862,12 +7898,12 @@
       </c>
       <c r="B214" s="5" t="inlineStr">
         <is>
-          <t>settings_disguise</t>
+          <t>shield_take_jeda</t>
         </is>
       </c>
       <c r="C214" s="5" t="inlineStr">
         <is>
-          <t>Pengaturan</t>
+          <t>Layar terkunci</t>
         </is>
       </c>
       <c r="D214" s="5" t="inlineStr">
@@ -7877,12 +7913,12 @@
       </c>
       <c r="E214" s="5" t="inlineStr">
         <is>
-          <t>Ikon &amp; nama samaran</t>
+          <t>Ambil jeda 60 detik</t>
         </is>
       </c>
       <c r="F214" s="5" t="inlineStr">
         <is>
-          <t>Disguised icon &amp; name</t>
+          <t>Take a 60-second pause</t>
         </is>
       </c>
       <c r="G214" s="5" t="inlineStr"/>
@@ -7895,12 +7931,12 @@
       </c>
       <c r="B215" s="5" t="inlineStr">
         <is>
-          <t>settings_hide_search</t>
+          <t>shield_close_app</t>
         </is>
       </c>
       <c r="C215" s="5" t="inlineStr">
         <is>
-          <t>Pengaturan</t>
+          <t>Layar terkunci</t>
         </is>
       </c>
       <c r="D215" s="5" t="inlineStr">
@@ -7910,19 +7946,15 @@
       </c>
       <c r="E215" s="5" t="inlineStr">
         <is>
-          <t>Sembunyikan dari pencarian HP</t>
+          <t>Tutup aplikasi</t>
         </is>
       </c>
       <c r="F215" s="5" t="inlineStr">
         <is>
-          <t>Hide from phone search</t>
-        </is>
-      </c>
-      <c r="G215" s="5" t="inlineStr">
-        <is>
-          <t>Android has no reliable API for this. Proposal: remove it, or replace it with 'Sembunyikan isi di layar Recent' / 'Hide content in Recents' (FLAG_SECURE).</t>
-        </is>
-      </c>
+          <t>Close the app</t>
+        </is>
+      </c>
+      <c r="G215" s="5" t="inlineStr"/>
       <c r="H215" s="6" t="inlineStr"/>
       <c r="I215" s="6" t="inlineStr"/>
     </row>
@@ -7932,12 +7964,12 @@
       </c>
       <c r="B216" s="7" t="inlineStr">
         <is>
-          <t>settings_hide_recents</t>
+          <t>shield_continue</t>
         </is>
       </c>
       <c r="C216" s="7" t="inlineStr">
         <is>
-          <t>Pengaturan</t>
+          <t>Layar terkunci</t>
         </is>
       </c>
       <c r="D216" s="7" t="inlineStr">
@@ -7947,17 +7979,17 @@
       </c>
       <c r="E216" s="7" t="inlineStr">
         <is>
-          <t>Sembunyikan isi di layar Recent</t>
+          <t>Tetap lanjutkan</t>
         </is>
       </c>
       <c r="F216" s="7" t="inlineStr">
         <is>
-          <t>Hide content in Recents</t>
+          <t>Continue anyway</t>
         </is>
       </c>
       <c r="G216" s="7" t="inlineStr">
         <is>
-          <t>Android replacement for the row above (FLAG_SECURE also blocks screenshots).</t>
+          <t>Needed for 'Pengingat lembut' mode, where the design has no continue button.</t>
         </is>
       </c>
       <c r="H216" s="6" t="inlineStr"/>
@@ -7969,12 +8001,12 @@
       </c>
       <c r="B217" s="5" t="inlineStr">
         <is>
-          <t>settings_group_journey</t>
+          <t>shield_note_gentle</t>
         </is>
       </c>
       <c r="C217" s="5" t="inlineStr">
         <is>
-          <t>Pengaturan</t>
+          <t>Layar terkunci</t>
         </is>
       </c>
       <c r="D217" s="5" t="inlineStr">
@@ -7984,12 +8016,12 @@
       </c>
       <c r="E217" s="5" t="inlineStr">
         <is>
-          <t>Perjalanan</t>
+          <t>Kamu tetap bisa melanjutkan jika memang perlu</t>
         </is>
       </c>
       <c r="F217" s="5" t="inlineStr">
         <is>
-          <t>Journey</t>
+          <t>You can still continue if you really need to</t>
         </is>
       </c>
       <c r="G217" s="5" t="inlineStr"/>
@@ -8002,12 +8034,12 @@
       </c>
       <c r="B218" s="5" t="inlineStr">
         <is>
-          <t>settings_target</t>
+          <t>shield_note_pause</t>
         </is>
       </c>
       <c r="C218" s="5" t="inlineStr">
         <is>
-          <t>Pengaturan</t>
+          <t>Layar terkunci</t>
         </is>
       </c>
       <c r="D218" s="5" t="inlineStr">
@@ -8017,12 +8049,12 @@
       </c>
       <c r="E218" s="5" t="inlineStr">
         <is>
-          <t>Target</t>
+          <t>Setelah jeda, aplikasi terbuka 5 menit</t>
         </is>
       </c>
       <c r="F218" s="5" t="inlineStr">
         <is>
-          <t>Goal</t>
+          <t>After the pause, the app opens for 5 minutes</t>
         </is>
       </c>
       <c r="G218" s="5" t="inlineStr"/>
@@ -8035,12 +8067,12 @@
       </c>
       <c r="B219" s="5" t="inlineStr">
         <is>
-          <t>settings_target_value</t>
+          <t>shield_note_full</t>
         </is>
       </c>
       <c r="C219" s="5" t="inlineStr">
         <is>
-          <t>Pengaturan</t>
+          <t>Layar terkunci</t>
         </is>
       </c>
       <c r="D219" s="5" t="inlineStr">
@@ -8050,19 +8082,15 @@
       </c>
       <c r="E219" s="5" t="inlineStr">
         <is>
-          <t>{n} hari</t>
+          <t>Terbuka lagi pukul {time}</t>
         </is>
       </c>
       <c r="F219" s="5" t="inlineStr">
         <is>
-          <t>{n} days</t>
-        </is>
-      </c>
-      <c r="G219" s="5" t="inlineStr">
-        <is>
-          <t>PLURAL in EN.</t>
-        </is>
-      </c>
+          <t>Opens again at {time}</t>
+        </is>
+      </c>
+      <c r="G219" s="5" t="inlineStr"/>
       <c r="H219" s="6" t="inlineStr"/>
       <c r="I219" s="6" t="inlineStr"/>
     </row>
@@ -8072,7 +8100,7 @@
       </c>
       <c r="B220" s="5" t="inlineStr">
         <is>
-          <t>settings_reminders</t>
+          <t>settings_title</t>
         </is>
       </c>
       <c r="C220" s="5" t="inlineStr">
@@ -8087,12 +8115,12 @@
       </c>
       <c r="E220" s="5" t="inlineStr">
         <is>
-          <t>Pengingat sholat &amp; dzikir</t>
+          <t>Pengaturan</t>
         </is>
       </c>
       <c r="F220" s="5" t="inlineStr">
         <is>
-          <t>Prayer &amp; dhikr reminders</t>
+          <t>Settings</t>
         </is>
       </c>
       <c r="G220" s="5" t="inlineStr"/>
@@ -8105,7 +8133,7 @@
       </c>
       <c r="B221" s="5" t="inlineStr">
         <is>
-          <t>settings_schedule</t>
+          <t>settings_profile_title</t>
         </is>
       </c>
       <c r="C221" s="5" t="inlineStr">
@@ -8120,12 +8148,12 @@
       </c>
       <c r="E221" s="5" t="inlineStr">
         <is>
-          <t>Jadwal waktu terjaga</t>
+          <t>Akun anonim</t>
         </is>
       </c>
       <c r="F221" s="5" t="inlineStr">
         <is>
-          <t>Guarded-hours schedule</t>
+          <t>Anonymous account</t>
         </is>
       </c>
       <c r="G221" s="5" t="inlineStr"/>
@@ -8138,7 +8166,7 @@
       </c>
       <c r="B222" s="5" t="inlineStr">
         <is>
-          <t>settings_group_data</t>
+          <t>settings_profile_sub</t>
         </is>
       </c>
       <c r="C222" s="5" t="inlineStr">
@@ -8153,12 +8181,12 @@
       </c>
       <c r="E222" s="5" t="inlineStr">
         <is>
-          <t>Data &amp; bantuan</t>
+          <t>Tanpa email · data hanya di HP ini</t>
         </is>
       </c>
       <c r="F222" s="5" t="inlineStr">
         <is>
-          <t>Data &amp; help</t>
+          <t>No email · data stays on this phone</t>
         </is>
       </c>
       <c r="G222" s="5" t="inlineStr"/>
@@ -8171,7 +8199,7 @@
       </c>
       <c r="B223" s="5" t="inlineStr">
         <is>
-          <t>settings_export_delete</t>
+          <t>settings_group_privacy</t>
         </is>
       </c>
       <c r="C223" s="5" t="inlineStr">
@@ -8186,12 +8214,12 @@
       </c>
       <c r="E223" s="5" t="inlineStr">
         <is>
-          <t>Ekspor &amp; hapus data</t>
+          <t>Privasi</t>
         </is>
       </c>
       <c r="F223" s="5" t="inlineStr">
         <is>
-          <t>Export &amp; delete data</t>
+          <t>Privacy</t>
         </is>
       </c>
       <c r="G223" s="5" t="inlineStr"/>
@@ -8199,76 +8227,72 @@
       <c r="I223" s="6" t="inlineStr"/>
     </row>
     <row r="224">
-      <c r="A224" s="5" t="n">
+      <c r="A224" s="8" t="n">
         <v>223</v>
       </c>
-      <c r="B224" s="5" t="inlineStr">
-        <is>
-          <t>settings_counselor</t>
-        </is>
-      </c>
-      <c r="C224" s="5" t="inlineStr">
+      <c r="B224" s="8" t="inlineStr">
+        <is>
+          <t>settings_pin_lock</t>
+        </is>
+      </c>
+      <c r="C224" s="8" t="inlineStr">
         <is>
           <t>Pengaturan</t>
         </is>
       </c>
-      <c r="D224" s="5" t="inlineStr">
-        <is>
-          <t>DESIGN</t>
-        </is>
-      </c>
-      <c r="E224" s="5" t="inlineStr">
-        <is>
-          <t>Bicara dengan konselor</t>
-        </is>
-      </c>
-      <c r="F224" s="5" t="inlineStr">
-        <is>
-          <t>Talk to a counselor</t>
-        </is>
-      </c>
-      <c r="G224" s="5" t="inlineStr">
-        <is>
-          <t>Where does it go? Needs a real contact or link before release.</t>
+      <c r="D224" s="8" t="inlineStr">
+        <is>
+          <t>ANDROID</t>
+        </is>
+      </c>
+      <c r="E224" s="8" t="inlineStr">
+        <is>
+          <t>Kunci dengan PIN &amp; sidik jari</t>
+        </is>
+      </c>
+      <c r="F224" s="8" t="inlineStr">
+        <is>
+          <t>Lock with PIN &amp; fingerprint</t>
+        </is>
+      </c>
+      <c r="G224" s="8" t="inlineStr">
+        <is>
+          <t>Original: '…&amp; Face ID'.</t>
         </is>
       </c>
       <c r="H224" s="6" t="inlineStr"/>
       <c r="I224" s="6" t="inlineStr"/>
     </row>
     <row r="225">
-      <c r="A225" s="7" t="n">
+      <c r="A225" s="5" t="n">
         <v>224</v>
       </c>
-      <c r="B225" s="7" t="inlineStr">
-        <is>
-          <t>counselor_placeholder</t>
-        </is>
-      </c>
-      <c r="C225" s="7" t="inlineStr">
+      <c r="B225" s="5" t="inlineStr">
+        <is>
+          <t>settings_disguise</t>
+        </is>
+      </c>
+      <c r="C225" s="5" t="inlineStr">
         <is>
           <t>Pengaturan</t>
         </is>
       </c>
-      <c r="D225" s="7" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="E225" s="7" t="inlineStr">
-        <is>
-          <t>Segera hadir. Kami sedang menyiapkan kontak konselor yang tepercaya.</t>
-        </is>
-      </c>
-      <c r="F225" s="7" t="inlineStr">
-        <is>
-          <t>Coming soon. We're preparing a trusted counselor contact.</t>
-        </is>
-      </c>
-      <c r="G225" s="7" t="inlineStr">
-        <is>
-          <t>Shown in the counselor sheet until a real contact or link exists.</t>
-        </is>
-      </c>
+      <c r="D225" s="5" t="inlineStr">
+        <is>
+          <t>DESIGN</t>
+        </is>
+      </c>
+      <c r="E225" s="5" t="inlineStr">
+        <is>
+          <t>Ikon &amp; nama samaran</t>
+        </is>
+      </c>
+      <c r="F225" s="5" t="inlineStr">
+        <is>
+          <t>Disguised icon &amp; name</t>
+        </is>
+      </c>
+      <c r="G225" s="5" t="inlineStr"/>
       <c r="H225" s="6" t="inlineStr"/>
       <c r="I225" s="6" t="inlineStr"/>
     </row>
@@ -8278,7 +8302,7 @@
       </c>
       <c r="B226" s="5" t="inlineStr">
         <is>
-          <t>settings_about</t>
+          <t>settings_hide_search</t>
         </is>
       </c>
       <c r="C226" s="5" t="inlineStr">
@@ -8293,15 +8317,19 @@
       </c>
       <c r="E226" s="5" t="inlineStr">
         <is>
-          <t>Tentang Izzah</t>
+          <t>Sembunyikan dari pencarian HP</t>
         </is>
       </c>
       <c r="F226" s="5" t="inlineStr">
         <is>
-          <t>About Izzah</t>
-        </is>
-      </c>
-      <c r="G226" s="5" t="inlineStr"/>
+          <t>Hide from phone search</t>
+        </is>
+      </c>
+      <c r="G226" s="5" t="inlineStr">
+        <is>
+          <t>Android has no reliable API for this. Proposal: remove it, or replace it with 'Sembunyikan isi di layar Recent' / 'Hide content in Recents' (FLAG_SECURE).</t>
+        </is>
+      </c>
       <c r="H226" s="6" t="inlineStr"/>
       <c r="I226" s="6" t="inlineStr"/>
     </row>
@@ -8311,7 +8339,7 @@
       </c>
       <c r="B227" s="7" t="inlineStr">
         <is>
-          <t>settings_language</t>
+          <t>settings_hide_recents</t>
         </is>
       </c>
       <c r="C227" s="7" t="inlineStr">
@@ -8326,124 +8354,120 @@
       </c>
       <c r="E227" s="7" t="inlineStr">
         <is>
-          <t>Bahasa</t>
+          <t>Sembunyikan isi di layar Recent</t>
         </is>
       </c>
       <c r="F227" s="7" t="inlineStr">
         <is>
-          <t>Language</t>
+          <t>Hide content in Recents</t>
         </is>
       </c>
       <c r="G227" s="7" t="inlineStr">
         <is>
-          <t>Language picker row, under Privasi or a new 'Umum' group.</t>
+          <t>Android replacement for the row above (FLAG_SECURE also blocks screenshots).</t>
         </is>
       </c>
       <c r="H227" s="6" t="inlineStr"/>
       <c r="I227" s="6" t="inlineStr"/>
     </row>
     <row r="228">
-      <c r="A228" s="7" t="n">
+      <c r="A228" s="5" t="n">
         <v>227</v>
       </c>
-      <c r="B228" s="7" t="inlineStr">
-        <is>
-          <t>language_system</t>
-        </is>
-      </c>
-      <c r="C228" s="7" t="inlineStr">
+      <c r="B228" s="5" t="inlineStr">
+        <is>
+          <t>settings_group_journey</t>
+        </is>
+      </c>
+      <c r="C228" s="5" t="inlineStr">
         <is>
           <t>Pengaturan</t>
         </is>
       </c>
-      <c r="D228" s="7" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="E228" s="7" t="inlineStr">
-        <is>
-          <t>Ikuti sistem</t>
-        </is>
-      </c>
-      <c r="F228" s="7" t="inlineStr">
-        <is>
-          <t>System default</t>
-        </is>
-      </c>
-      <c r="G228" s="7" t="inlineStr"/>
+      <c r="D228" s="5" t="inlineStr">
+        <is>
+          <t>DESIGN</t>
+        </is>
+      </c>
+      <c r="E228" s="5" t="inlineStr">
+        <is>
+          <t>Perjalanan</t>
+        </is>
+      </c>
+      <c r="F228" s="5" t="inlineStr">
+        <is>
+          <t>Journey</t>
+        </is>
+      </c>
+      <c r="G228" s="5" t="inlineStr"/>
       <c r="H228" s="6" t="inlineStr"/>
       <c r="I228" s="6" t="inlineStr"/>
     </row>
     <row r="229">
-      <c r="A229" s="7" t="n">
+      <c r="A229" s="5" t="n">
         <v>228</v>
       </c>
-      <c r="B229" s="7" t="inlineStr">
-        <is>
-          <t>language_id</t>
-        </is>
-      </c>
-      <c r="C229" s="7" t="inlineStr">
+      <c r="B229" s="5" t="inlineStr">
+        <is>
+          <t>settings_target</t>
+        </is>
+      </c>
+      <c r="C229" s="5" t="inlineStr">
         <is>
           <t>Pengaturan</t>
         </is>
       </c>
-      <c r="D229" s="7" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="E229" s="7" t="inlineStr">
-        <is>
-          <t>Bahasa Indonesia</t>
-        </is>
-      </c>
-      <c r="F229" s="7" t="inlineStr">
-        <is>
-          <t>Bahasa Indonesia</t>
-        </is>
-      </c>
-      <c r="G229" s="7" t="inlineStr">
-        <is>
-          <t>Always shown in its own language.</t>
-        </is>
-      </c>
+      <c r="D229" s="5" t="inlineStr">
+        <is>
+          <t>DESIGN</t>
+        </is>
+      </c>
+      <c r="E229" s="5" t="inlineStr">
+        <is>
+          <t>Target</t>
+        </is>
+      </c>
+      <c r="F229" s="5" t="inlineStr">
+        <is>
+          <t>Goal</t>
+        </is>
+      </c>
+      <c r="G229" s="5" t="inlineStr"/>
       <c r="H229" s="6" t="inlineStr"/>
       <c r="I229" s="6" t="inlineStr"/>
     </row>
     <row r="230">
-      <c r="A230" s="7" t="n">
+      <c r="A230" s="5" t="n">
         <v>229</v>
       </c>
-      <c r="B230" s="7" t="inlineStr">
-        <is>
-          <t>language_en</t>
-        </is>
-      </c>
-      <c r="C230" s="7" t="inlineStr">
+      <c r="B230" s="5" t="inlineStr">
+        <is>
+          <t>settings_target_value</t>
+        </is>
+      </c>
+      <c r="C230" s="5" t="inlineStr">
         <is>
           <t>Pengaturan</t>
         </is>
       </c>
-      <c r="D230" s="7" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="E230" s="7" t="inlineStr">
-        <is>
-          <t>English</t>
-        </is>
-      </c>
-      <c r="F230" s="7" t="inlineStr">
-        <is>
-          <t>English</t>
-        </is>
-      </c>
-      <c r="G230" s="7" t="inlineStr">
-        <is>
-          <t>Always shown in its own language.</t>
+      <c r="D230" s="5" t="inlineStr">
+        <is>
+          <t>DESIGN</t>
+        </is>
+      </c>
+      <c r="E230" s="5" t="inlineStr">
+        <is>
+          <t>{n} hari</t>
+        </is>
+      </c>
+      <c r="F230" s="5" t="inlineStr">
+        <is>
+          <t>{n} days</t>
+        </is>
+      </c>
+      <c r="G230" s="5" t="inlineStr">
+        <is>
+          <t>PLURAL in EN.</t>
         </is>
       </c>
       <c r="H230" s="6" t="inlineStr"/>
@@ -8455,12 +8479,12 @@
       </c>
       <c r="B231" s="5" t="inlineStr">
         <is>
-          <t>disguise_title</t>
+          <t>settings_reminders</t>
         </is>
       </c>
       <c r="C231" s="5" t="inlineStr">
         <is>
-          <t>Ikon samaran</t>
+          <t>Pengaturan</t>
         </is>
       </c>
       <c r="D231" s="5" t="inlineStr">
@@ -8470,12 +8494,12 @@
       </c>
       <c r="E231" s="5" t="inlineStr">
         <is>
-          <t>Ikon samaran</t>
+          <t>Pengingat sholat &amp; dzikir</t>
         </is>
       </c>
       <c r="F231" s="5" t="inlineStr">
         <is>
-          <t>Disguised icon</t>
+          <t>Prayer &amp; dhikr reminders</t>
         </is>
       </c>
       <c r="G231" s="5" t="inlineStr"/>
@@ -8488,12 +8512,12 @@
       </c>
       <c r="B232" s="5" t="inlineStr">
         <is>
-          <t>disguise_desc</t>
+          <t>settings_schedule</t>
         </is>
       </c>
       <c r="C232" s="5" t="inlineStr">
         <is>
-          <t>Ikon samaran</t>
+          <t>Pengaturan</t>
         </is>
       </c>
       <c r="D232" s="5" t="inlineStr">
@@ -8503,12 +8527,12 @@
       </c>
       <c r="E232" s="5" t="inlineStr">
         <is>
-          <t>Ganti ikon dan nama di layar HP supaya tidak menarik perhatian.</t>
+          <t>Jadwal waktu terjaga</t>
         </is>
       </c>
       <c r="F232" s="5" t="inlineStr">
         <is>
-          <t>Change the icon and name on your home screen so it doesn't draw attention.</t>
+          <t>Guarded-hours schedule</t>
         </is>
       </c>
       <c r="G232" s="5" t="inlineStr"/>
@@ -8521,12 +8545,12 @@
       </c>
       <c r="B233" s="5" t="inlineStr">
         <is>
-          <t>disguise_izzah</t>
+          <t>settings_group_data</t>
         </is>
       </c>
       <c r="C233" s="5" t="inlineStr">
         <is>
-          <t>Ikon samaran</t>
+          <t>Pengaturan</t>
         </is>
       </c>
       <c r="D233" s="5" t="inlineStr">
@@ -8536,12 +8560,12 @@
       </c>
       <c r="E233" s="5" t="inlineStr">
         <is>
-          <t>Izzah</t>
+          <t>Data &amp; bantuan</t>
         </is>
       </c>
       <c r="F233" s="5" t="inlineStr">
         <is>
-          <t>Izzah</t>
+          <t>Data &amp; help</t>
         </is>
       </c>
       <c r="G233" s="5" t="inlineStr"/>
@@ -8554,12 +8578,12 @@
       </c>
       <c r="B234" s="5" t="inlineStr">
         <is>
-          <t>disguise_steps</t>
+          <t>settings_export_delete</t>
         </is>
       </c>
       <c r="C234" s="5" t="inlineStr">
         <is>
-          <t>Ikon samaran</t>
+          <t>Pengaturan</t>
         </is>
       </c>
       <c r="D234" s="5" t="inlineStr">
@@ -8569,19 +8593,15 @@
       </c>
       <c r="E234" s="5" t="inlineStr">
         <is>
-          <t>Langkah</t>
+          <t>Ekspor &amp; hapus data</t>
         </is>
       </c>
       <c r="F234" s="5" t="inlineStr">
         <is>
-          <t>Steps</t>
-        </is>
-      </c>
-      <c r="G234" s="5" t="inlineStr">
-        <is>
-          <t>This becomes the launcher label, so it's localized too.</t>
-        </is>
-      </c>
+          <t>Export &amp; delete data</t>
+        </is>
+      </c>
+      <c r="G234" s="5" t="inlineStr"/>
       <c r="H234" s="6" t="inlineStr"/>
       <c r="I234" s="6" t="inlineStr"/>
     </row>
@@ -8591,12 +8611,12 @@
       </c>
       <c r="B235" s="5" t="inlineStr">
         <is>
-          <t>disguise_focus</t>
+          <t>settings_counselor</t>
         </is>
       </c>
       <c r="C235" s="5" t="inlineStr">
         <is>
-          <t>Ikon samaran</t>
+          <t>Pengaturan</t>
         </is>
       </c>
       <c r="D235" s="5" t="inlineStr">
@@ -8606,217 +8626,233 @@
       </c>
       <c r="E235" s="5" t="inlineStr">
         <is>
-          <t>Fokus</t>
+          <t>Bicara dengan konselor</t>
         </is>
       </c>
       <c r="F235" s="5" t="inlineStr">
         <is>
-          <t>Focus</t>
-        </is>
-      </c>
-      <c r="G235" s="5" t="inlineStr"/>
+          <t>Talk to a counselor</t>
+        </is>
+      </c>
+      <c r="G235" s="5" t="inlineStr">
+        <is>
+          <t>Where does it go? Needs a real contact or link before release.</t>
+        </is>
+      </c>
       <c r="H235" s="6" t="inlineStr"/>
       <c r="I235" s="6" t="inlineStr"/>
     </row>
     <row r="236">
-      <c r="A236" s="5" t="n">
+      <c r="A236" s="7" t="n">
         <v>235</v>
       </c>
-      <c r="B236" s="5" t="inlineStr">
-        <is>
-          <t>disguise_notes</t>
-        </is>
-      </c>
-      <c r="C236" s="5" t="inlineStr">
-        <is>
-          <t>Ikon samaran</t>
-        </is>
-      </c>
-      <c r="D236" s="5" t="inlineStr">
-        <is>
-          <t>DESIGN</t>
-        </is>
-      </c>
-      <c r="E236" s="5" t="inlineStr">
-        <is>
-          <t>Catatan</t>
-        </is>
-      </c>
-      <c r="F236" s="5" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-      <c r="G236" s="5" t="inlineStr"/>
+      <c r="B236" s="7" t="inlineStr">
+        <is>
+          <t>counselor_placeholder</t>
+        </is>
+      </c>
+      <c r="C236" s="7" t="inlineStr">
+        <is>
+          <t>Pengaturan</t>
+        </is>
+      </c>
+      <c r="D236" s="7" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="E236" s="7" t="inlineStr">
+        <is>
+          <t>Segera hadir. Kami sedang menyiapkan kontak konselor yang tepercaya.</t>
+        </is>
+      </c>
+      <c r="F236" s="7" t="inlineStr">
+        <is>
+          <t>Coming soon. We're preparing a trusted counselor contact.</t>
+        </is>
+      </c>
+      <c r="G236" s="7" t="inlineStr">
+        <is>
+          <t>Shown in the counselor sheet until a real contact or link exists.</t>
+        </is>
+      </c>
       <c r="H236" s="6" t="inlineStr"/>
       <c r="I236" s="6" t="inlineStr"/>
     </row>
     <row r="237">
-      <c r="A237" s="8" t="n">
+      <c r="A237" s="5" t="n">
         <v>236</v>
       </c>
-      <c r="B237" s="8" t="inlineStr">
-        <is>
-          <t>disguise_footer</t>
-        </is>
-      </c>
-      <c r="C237" s="8" t="inlineStr">
-        <is>
-          <t>Ikon samaran</t>
-        </is>
-      </c>
-      <c r="D237" s="8" t="inlineStr">
-        <is>
-          <t>ANDROID</t>
-        </is>
-      </c>
-      <c r="E237" s="8" t="inlineStr">
-        <is>
-          <t>Nama di notifikasi tetap “Izzah”, tapi isinya selalu netral.</t>
-        </is>
-      </c>
-      <c r="F237" s="8" t="inlineStr">
-        <is>
-          <t>Notifications still show “Izzah”, but their content is always neutral.</t>
-        </is>
-      </c>
-      <c r="G237" s="8" t="inlineStr">
-        <is>
-          <t>Original: 'Notifikasi akan memakai nama yang sama.' Android always shows the application label in notifications; an activity-alias can't change it.</t>
-        </is>
-      </c>
+      <c r="B237" s="5" t="inlineStr">
+        <is>
+          <t>settings_about</t>
+        </is>
+      </c>
+      <c r="C237" s="5" t="inlineStr">
+        <is>
+          <t>Pengaturan</t>
+        </is>
+      </c>
+      <c r="D237" s="5" t="inlineStr">
+        <is>
+          <t>DESIGN</t>
+        </is>
+      </c>
+      <c r="E237" s="5" t="inlineStr">
+        <is>
+          <t>Tentang Izzah</t>
+        </is>
+      </c>
+      <c r="F237" s="5" t="inlineStr">
+        <is>
+          <t>About Izzah</t>
+        </is>
+      </c>
+      <c r="G237" s="5" t="inlineStr"/>
       <c r="H237" s="6" t="inlineStr"/>
       <c r="I237" s="6" t="inlineStr"/>
     </row>
     <row r="238">
-      <c r="A238" s="5" t="n">
+      <c r="A238" s="7" t="n">
         <v>237</v>
       </c>
-      <c r="B238" s="5" t="inlineStr">
-        <is>
-          <t>data_title</t>
-        </is>
-      </c>
-      <c r="C238" s="5" t="inlineStr">
-        <is>
-          <t>Datamu</t>
-        </is>
-      </c>
-      <c r="D238" s="5" t="inlineStr">
-        <is>
-          <t>DESIGN</t>
-        </is>
-      </c>
-      <c r="E238" s="5" t="inlineStr">
-        <is>
-          <t>Datamu</t>
-        </is>
-      </c>
-      <c r="F238" s="5" t="inlineStr">
-        <is>
-          <t>Your data</t>
-        </is>
-      </c>
-      <c r="G238" s="5" t="inlineStr"/>
+      <c r="B238" s="7" t="inlineStr">
+        <is>
+          <t>settings_language</t>
+        </is>
+      </c>
+      <c r="C238" s="7" t="inlineStr">
+        <is>
+          <t>Pengaturan</t>
+        </is>
+      </c>
+      <c r="D238" s="7" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="E238" s="7" t="inlineStr">
+        <is>
+          <t>Bahasa</t>
+        </is>
+      </c>
+      <c r="F238" s="7" t="inlineStr">
+        <is>
+          <t>Language</t>
+        </is>
+      </c>
+      <c r="G238" s="7" t="inlineStr">
+        <is>
+          <t>Language picker row, under Privasi or a new 'Umum' group.</t>
+        </is>
+      </c>
       <c r="H238" s="6" t="inlineStr"/>
       <c r="I238" s="6" t="inlineStr"/>
     </row>
     <row r="239">
-      <c r="A239" s="5" t="n">
+      <c r="A239" s="7" t="n">
         <v>238</v>
       </c>
-      <c r="B239" s="5" t="inlineStr">
-        <is>
-          <t>data_desc</t>
-        </is>
-      </c>
-      <c r="C239" s="5" t="inlineStr">
-        <is>
-          <t>Datamu</t>
-        </is>
-      </c>
-      <c r="D239" s="5" t="inlineStr">
-        <is>
-          <t>DESIGN</t>
-        </is>
-      </c>
-      <c r="E239" s="5" t="inlineStr">
-        <is>
-          <t>Semua tersimpan di HP ini. Tidak ada di server kami.</t>
-        </is>
-      </c>
-      <c r="F239" s="5" t="inlineStr">
-        <is>
-          <t>Everything is stored on this phone. Nothing is on our servers.</t>
-        </is>
-      </c>
-      <c r="G239" s="5" t="inlineStr"/>
+      <c r="B239" s="7" t="inlineStr">
+        <is>
+          <t>language_system</t>
+        </is>
+      </c>
+      <c r="C239" s="7" t="inlineStr">
+        <is>
+          <t>Pengaturan</t>
+        </is>
+      </c>
+      <c r="D239" s="7" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="E239" s="7" t="inlineStr">
+        <is>
+          <t>Ikuti sistem</t>
+        </is>
+      </c>
+      <c r="F239" s="7" t="inlineStr">
+        <is>
+          <t>System default</t>
+        </is>
+      </c>
+      <c r="G239" s="7" t="inlineStr"/>
       <c r="H239" s="6" t="inlineStr"/>
       <c r="I239" s="6" t="inlineStr"/>
     </row>
     <row r="240">
-      <c r="A240" s="5" t="n">
+      <c r="A240" s="7" t="n">
         <v>239</v>
       </c>
-      <c r="B240" s="5" t="inlineStr">
-        <is>
-          <t>data_export_title</t>
-        </is>
-      </c>
-      <c r="C240" s="5" t="inlineStr">
-        <is>
-          <t>Datamu</t>
-        </is>
-      </c>
-      <c r="D240" s="5" t="inlineStr">
-        <is>
-          <t>DESIGN</t>
-        </is>
-      </c>
-      <c r="E240" s="5" t="inlineStr">
-        <is>
-          <t>Ekspor cadangan</t>
-        </is>
-      </c>
-      <c r="F240" s="5" t="inlineStr">
-        <is>
-          <t>Export a backup</t>
-        </is>
-      </c>
-      <c r="G240" s="5" t="inlineStr"/>
+      <c r="B240" s="7" t="inlineStr">
+        <is>
+          <t>language_id</t>
+        </is>
+      </c>
+      <c r="C240" s="7" t="inlineStr">
+        <is>
+          <t>Pengaturan</t>
+        </is>
+      </c>
+      <c r="D240" s="7" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="E240" s="7" t="inlineStr">
+        <is>
+          <t>Bahasa Indonesia</t>
+        </is>
+      </c>
+      <c r="F240" s="7" t="inlineStr">
+        <is>
+          <t>Bahasa Indonesia</t>
+        </is>
+      </c>
+      <c r="G240" s="7" t="inlineStr">
+        <is>
+          <t>Always shown in its own language.</t>
+        </is>
+      </c>
       <c r="H240" s="6" t="inlineStr"/>
       <c r="I240" s="6" t="inlineStr"/>
     </row>
     <row r="241">
-      <c r="A241" s="5" t="n">
+      <c r="A241" s="7" t="n">
         <v>240</v>
       </c>
-      <c r="B241" s="5" t="inlineStr">
-        <is>
-          <t>data_export_desc</t>
-        </is>
-      </c>
-      <c r="C241" s="5" t="inlineStr">
-        <is>
-          <t>Datamu</t>
-        </is>
-      </c>
-      <c r="D241" s="5" t="inlineStr">
-        <is>
-          <t>DESIGN</t>
-        </is>
-      </c>
-      <c r="E241" s="5" t="inlineStr">
-        <is>
-          <t>File terenkripsi dengan PIN-mu. Pakai saat pindah HP.</t>
-        </is>
-      </c>
-      <c r="F241" s="5" t="inlineStr">
-        <is>
-          <t>A file encrypted with your PIN. Use it when you switch phones.</t>
-        </is>
-      </c>
-      <c r="G241" s="5" t="inlineStr"/>
+      <c r="B241" s="7" t="inlineStr">
+        <is>
+          <t>language_en</t>
+        </is>
+      </c>
+      <c r="C241" s="7" t="inlineStr">
+        <is>
+          <t>Pengaturan</t>
+        </is>
+      </c>
+      <c r="D241" s="7" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="E241" s="7" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F241" s="7" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="G241" s="7" t="inlineStr">
+        <is>
+          <t>Always shown in its own language.</t>
+        </is>
+      </c>
       <c r="H241" s="6" t="inlineStr"/>
       <c r="I241" s="6" t="inlineStr"/>
     </row>
@@ -8826,12 +8862,12 @@
       </c>
       <c r="B242" s="5" t="inlineStr">
         <is>
-          <t>data_export_cta</t>
+          <t>disguise_title</t>
         </is>
       </c>
       <c r="C242" s="5" t="inlineStr">
         <is>
-          <t>Datamu</t>
+          <t>Ikon samaran</t>
         </is>
       </c>
       <c r="D242" s="5" t="inlineStr">
@@ -8841,12 +8877,12 @@
       </c>
       <c r="E242" s="5" t="inlineStr">
         <is>
-          <t>Buat file cadangan</t>
+          <t>Ikon samaran</t>
         </is>
       </c>
       <c r="F242" s="5" t="inlineStr">
         <is>
-          <t>Create backup file</t>
+          <t>Disguised icon</t>
         </is>
       </c>
       <c r="G242" s="5" t="inlineStr"/>
@@ -8854,107 +8890,103 @@
       <c r="I242" s="6" t="inlineStr"/>
     </row>
     <row r="243">
-      <c r="A243" s="7" t="n">
+      <c r="A243" s="5" t="n">
         <v>242</v>
       </c>
-      <c r="B243" s="7" t="inlineStr">
-        <is>
-          <t>data_import_wrong_pin</t>
-        </is>
-      </c>
-      <c r="C243" s="7" t="inlineStr">
-        <is>
-          <t>Datamu</t>
-        </is>
-      </c>
-      <c r="D243" s="7" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="E243" s="7" t="inlineStr">
-        <is>
-          <t>PIN cadangan tidak cocok.</t>
-        </is>
-      </c>
-      <c r="F243" s="7" t="inlineStr">
-        <is>
-          <t>The backup PIN doesn't match.</t>
-        </is>
-      </c>
-      <c r="G243" s="7" t="inlineStr"/>
+      <c r="B243" s="5" t="inlineStr">
+        <is>
+          <t>disguise_desc</t>
+        </is>
+      </c>
+      <c r="C243" s="5" t="inlineStr">
+        <is>
+          <t>Ikon samaran</t>
+        </is>
+      </c>
+      <c r="D243" s="5" t="inlineStr">
+        <is>
+          <t>DESIGN</t>
+        </is>
+      </c>
+      <c r="E243" s="5" t="inlineStr">
+        <is>
+          <t>Ganti ikon dan nama di layar HP supaya tidak menarik perhatian.</t>
+        </is>
+      </c>
+      <c r="F243" s="5" t="inlineStr">
+        <is>
+          <t>Change the icon and name on your home screen so it doesn't draw attention.</t>
+        </is>
+      </c>
+      <c r="G243" s="5" t="inlineStr"/>
       <c r="H243" s="6" t="inlineStr"/>
       <c r="I243" s="6" t="inlineStr"/>
     </row>
     <row r="244">
-      <c r="A244" s="7" t="n">
+      <c r="A244" s="5" t="n">
         <v>243</v>
       </c>
-      <c r="B244" s="7" t="inlineStr">
-        <is>
-          <t>data_export_done</t>
-        </is>
-      </c>
-      <c r="C244" s="7" t="inlineStr">
-        <is>
-          <t>Datamu</t>
-        </is>
-      </c>
-      <c r="D244" s="7" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="E244" s="7" t="inlineStr">
-        <is>
-          <t>Cadangan tersimpan.</t>
-        </is>
-      </c>
-      <c r="F244" s="7" t="inlineStr">
-        <is>
-          <t>Backup saved.</t>
-        </is>
-      </c>
-      <c r="G244" s="7" t="inlineStr">
-        <is>
-          <t>Toast after the system save dialog.</t>
-        </is>
-      </c>
+      <c r="B244" s="5" t="inlineStr">
+        <is>
+          <t>disguise_izzah</t>
+        </is>
+      </c>
+      <c r="C244" s="5" t="inlineStr">
+        <is>
+          <t>Ikon samaran</t>
+        </is>
+      </c>
+      <c r="D244" s="5" t="inlineStr">
+        <is>
+          <t>DESIGN</t>
+        </is>
+      </c>
+      <c r="E244" s="5" t="inlineStr">
+        <is>
+          <t>Izzah</t>
+        </is>
+      </c>
+      <c r="F244" s="5" t="inlineStr">
+        <is>
+          <t>Izzah</t>
+        </is>
+      </c>
+      <c r="G244" s="5" t="inlineStr"/>
       <c r="H244" s="6" t="inlineStr"/>
       <c r="I244" s="6" t="inlineStr"/>
     </row>
     <row r="245">
-      <c r="A245" s="7" t="n">
+      <c r="A245" s="5" t="n">
         <v>244</v>
       </c>
-      <c r="B245" s="7" t="inlineStr">
-        <is>
-          <t>data_import_cta</t>
-        </is>
-      </c>
-      <c r="C245" s="7" t="inlineStr">
-        <is>
-          <t>Datamu</t>
-        </is>
-      </c>
-      <c r="D245" s="7" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="E245" s="7" t="inlineStr">
-        <is>
-          <t>Pulihkan dari cadangan</t>
-        </is>
-      </c>
-      <c r="F245" s="7" t="inlineStr">
-        <is>
-          <t>Restore from backup</t>
-        </is>
-      </c>
-      <c r="G245" s="7" t="inlineStr">
-        <is>
-          <t>Without this, the export is useless on a new phone. Proposed for v1.</t>
+      <c r="B245" s="5" t="inlineStr">
+        <is>
+          <t>disguise_steps</t>
+        </is>
+      </c>
+      <c r="C245" s="5" t="inlineStr">
+        <is>
+          <t>Ikon samaran</t>
+        </is>
+      </c>
+      <c r="D245" s="5" t="inlineStr">
+        <is>
+          <t>DESIGN</t>
+        </is>
+      </c>
+      <c r="E245" s="5" t="inlineStr">
+        <is>
+          <t>Langkah</t>
+        </is>
+      </c>
+      <c r="F245" s="5" t="inlineStr">
+        <is>
+          <t>Steps</t>
+        </is>
+      </c>
+      <c r="G245" s="5" t="inlineStr">
+        <is>
+          <t>This becomes the launcher label, so it's localized too.</t>
         </is>
       </c>
       <c r="H245" s="6" t="inlineStr"/>
@@ -8966,12 +8998,12 @@
       </c>
       <c r="B246" s="5" t="inlineStr">
         <is>
-          <t>data_delete_title</t>
+          <t>disguise_focus</t>
         </is>
       </c>
       <c r="C246" s="5" t="inlineStr">
         <is>
-          <t>Datamu</t>
+          <t>Ikon samaran</t>
         </is>
       </c>
       <c r="D246" s="5" t="inlineStr">
@@ -8981,12 +9013,12 @@
       </c>
       <c r="E246" s="5" t="inlineStr">
         <is>
-          <t>Hapus semua data</t>
+          <t>Fokus</t>
         </is>
       </c>
       <c r="F246" s="5" t="inlineStr">
         <is>
-          <t>Delete all data</t>
+          <t>Focus</t>
         </is>
       </c>
       <c r="G246" s="5" t="inlineStr"/>
@@ -8999,12 +9031,12 @@
       </c>
       <c r="B247" s="5" t="inlineStr">
         <is>
-          <t>data_delete_desc</t>
+          <t>disguise_notes</t>
         </is>
       </c>
       <c r="C247" s="5" t="inlineStr">
         <is>
-          <t>Datamu</t>
+          <t>Ikon samaran</t>
         </is>
       </c>
       <c r="D247" s="5" t="inlineStr">
@@ -9014,12 +9046,12 @@
       </c>
       <c r="E247" s="5" t="inlineStr">
         <is>
-          <t>Progres, jurnal, dan pengaturan akan hilang permanen.</t>
+          <t>Catatan</t>
         </is>
       </c>
       <c r="F247" s="5" t="inlineStr">
         <is>
-          <t>Your progress, journal and settings will be permanently erased.</t>
+          <t>Notes</t>
         </is>
       </c>
       <c r="G247" s="5" t="inlineStr"/>
@@ -9027,35 +9059,39 @@
       <c r="I247" s="6" t="inlineStr"/>
     </row>
     <row r="248">
-      <c r="A248" s="5" t="n">
+      <c r="A248" s="8" t="n">
         <v>247</v>
       </c>
-      <c r="B248" s="5" t="inlineStr">
-        <is>
-          <t>data_delete_cta</t>
-        </is>
-      </c>
-      <c r="C248" s="5" t="inlineStr">
-        <is>
-          <t>Datamu</t>
-        </is>
-      </c>
-      <c r="D248" s="5" t="inlineStr">
-        <is>
-          <t>DESIGN</t>
-        </is>
-      </c>
-      <c r="E248" s="5" t="inlineStr">
-        <is>
-          <t>Hapus data</t>
-        </is>
-      </c>
-      <c r="F248" s="5" t="inlineStr">
-        <is>
-          <t>Delete data</t>
-        </is>
-      </c>
-      <c r="G248" s="5" t="inlineStr"/>
+      <c r="B248" s="8" t="inlineStr">
+        <is>
+          <t>disguise_footer</t>
+        </is>
+      </c>
+      <c r="C248" s="8" t="inlineStr">
+        <is>
+          <t>Ikon samaran</t>
+        </is>
+      </c>
+      <c r="D248" s="8" t="inlineStr">
+        <is>
+          <t>ANDROID</t>
+        </is>
+      </c>
+      <c r="E248" s="8" t="inlineStr">
+        <is>
+          <t>Nama di notifikasi tetap “Izzah”, tapi isinya selalu netral.</t>
+        </is>
+      </c>
+      <c r="F248" s="8" t="inlineStr">
+        <is>
+          <t>Notifications still show “Izzah”, but their content is always neutral.</t>
+        </is>
+      </c>
+      <c r="G248" s="8" t="inlineStr">
+        <is>
+          <t>Original: 'Notifikasi akan memakai nama yang sama.' Android always shows the application label in notifications; an activity-alias can't change it.</t>
+        </is>
+      </c>
       <c r="H248" s="6" t="inlineStr"/>
       <c r="I248" s="6" t="inlineStr"/>
     </row>
@@ -9065,12 +9101,12 @@
       </c>
       <c r="B249" s="5" t="inlineStr">
         <is>
-          <t>delete_sheet_title</t>
+          <t>data_title</t>
         </is>
       </c>
       <c r="C249" s="5" t="inlineStr">
         <is>
-          <t>Hapus (sheet)</t>
+          <t>Datamu</t>
         </is>
       </c>
       <c r="D249" s="5" t="inlineStr">
@@ -9080,12 +9116,12 @@
       </c>
       <c r="E249" s="5" t="inlineStr">
         <is>
-          <t>Yakin hapus semua?</t>
+          <t>Datamu</t>
         </is>
       </c>
       <c r="F249" s="5" t="inlineStr">
         <is>
-          <t>Delete everything?</t>
+          <t>Your data</t>
         </is>
       </c>
       <c r="G249" s="5" t="inlineStr"/>
@@ -9098,12 +9134,12 @@
       </c>
       <c r="B250" s="5" t="inlineStr">
         <is>
-          <t>delete_sheet_body</t>
+          <t>data_desc</t>
         </is>
       </c>
       <c r="C250" s="5" t="inlineStr">
         <is>
-          <t>Hapus (sheet)</t>
+          <t>Datamu</t>
         </is>
       </c>
       <c r="D250" s="5" t="inlineStr">
@@ -9113,12 +9149,12 @@
       </c>
       <c r="E250" s="5" t="inlineStr">
         <is>
-          <t>Ini tidak bisa dibatalkan. Kalau hanya ingin istirahat, kamu bisa menjeda pengingat saja.</t>
+          <t>Semua tersimpan di HP ini. Tidak ada di server kami.</t>
         </is>
       </c>
       <c r="F250" s="5" t="inlineStr">
         <is>
-          <t>This can't be undone. If you just need a break, you can pause the reminders instead.</t>
+          <t>Everything is stored on this phone. Nothing is on our servers.</t>
         </is>
       </c>
       <c r="G250" s="5" t="inlineStr"/>
@@ -9131,12 +9167,12 @@
       </c>
       <c r="B251" s="5" t="inlineStr">
         <is>
-          <t>delete_sheet_confirm</t>
+          <t>data_export_title</t>
         </is>
       </c>
       <c r="C251" s="5" t="inlineStr">
         <is>
-          <t>Hapus (sheet)</t>
+          <t>Datamu</t>
         </is>
       </c>
       <c r="D251" s="5" t="inlineStr">
@@ -9146,12 +9182,12 @@
       </c>
       <c r="E251" s="5" t="inlineStr">
         <is>
-          <t>Ya, hapus semuanya</t>
+          <t>Ekspor cadangan</t>
         </is>
       </c>
       <c r="F251" s="5" t="inlineStr">
         <is>
-          <t>Yes, delete everything</t>
+          <t>Export a backup</t>
         </is>
       </c>
       <c r="G251" s="5" t="inlineStr"/>
@@ -9164,12 +9200,12 @@
       </c>
       <c r="B252" s="5" t="inlineStr">
         <is>
-          <t>common_cancel</t>
+          <t>data_export_desc</t>
         </is>
       </c>
       <c r="C252" s="5" t="inlineStr">
         <is>
-          <t>Hapus (sheet)</t>
+          <t>Datamu</t>
         </is>
       </c>
       <c r="D252" s="5" t="inlineStr">
@@ -9179,12 +9215,12 @@
       </c>
       <c r="E252" s="5" t="inlineStr">
         <is>
-          <t>Batal</t>
+          <t>File terenkripsi dengan PIN-mu. Pakai saat pindah HP.</t>
         </is>
       </c>
       <c r="F252" s="5" t="inlineStr">
         <is>
-          <t>Cancel</t>
+          <t>A file encrypted with your PIN. Use it when you switch phones.</t>
         </is>
       </c>
       <c r="G252" s="5" t="inlineStr"/>
@@ -9197,12 +9233,12 @@
       </c>
       <c r="B253" s="5" t="inlineStr">
         <is>
-          <t>unlock_title</t>
+          <t>data_export_cta</t>
         </is>
       </c>
       <c r="C253" s="5" t="inlineStr">
         <is>
-          <t>Buka dengan PIN</t>
+          <t>Datamu</t>
         </is>
       </c>
       <c r="D253" s="5" t="inlineStr">
@@ -9212,12 +9248,12 @@
       </c>
       <c r="E253" s="5" t="inlineStr">
         <is>
-          <t>Masukkan PIN</t>
+          <t>Buat file cadangan</t>
         </is>
       </c>
       <c r="F253" s="5" t="inlineStr">
         <is>
-          <t>Enter your PIN</t>
+          <t>Create backup file</t>
         </is>
       </c>
       <c r="G253" s="5" t="inlineStr"/>
@@ -9225,35 +9261,35 @@
       <c r="I253" s="6" t="inlineStr"/>
     </row>
     <row r="254">
-      <c r="A254" s="5" t="n">
+      <c r="A254" s="7" t="n">
         <v>253</v>
       </c>
-      <c r="B254" s="5" t="inlineStr">
-        <is>
-          <t>unlock_subtitle</t>
-        </is>
-      </c>
-      <c r="C254" s="5" t="inlineStr">
-        <is>
-          <t>Buka dengan PIN</t>
-        </is>
-      </c>
-      <c r="D254" s="5" t="inlineStr">
-        <is>
-          <t>DESIGN</t>
-        </is>
-      </c>
-      <c r="E254" s="5" t="inlineStr">
-        <is>
-          <t>Assalamu’alaikum. Selamat datang kembali.</t>
-        </is>
-      </c>
-      <c r="F254" s="5" t="inlineStr">
-        <is>
-          <t>Assalamu’alaikum. Welcome back.</t>
-        </is>
-      </c>
-      <c r="G254" s="5" t="inlineStr"/>
+      <c r="B254" s="7" t="inlineStr">
+        <is>
+          <t>data_import_wrong_pin</t>
+        </is>
+      </c>
+      <c r="C254" s="7" t="inlineStr">
+        <is>
+          <t>Datamu</t>
+        </is>
+      </c>
+      <c r="D254" s="7" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="E254" s="7" t="inlineStr">
+        <is>
+          <t>PIN cadangan tidak cocok.</t>
+        </is>
+      </c>
+      <c r="F254" s="7" t="inlineStr">
+        <is>
+          <t>The backup PIN doesn't match.</t>
+        </is>
+      </c>
+      <c r="G254" s="7" t="inlineStr"/>
       <c r="H254" s="6" t="inlineStr"/>
       <c r="I254" s="6" t="inlineStr"/>
     </row>
@@ -9263,12 +9299,12 @@
       </c>
       <c r="B255" s="7" t="inlineStr">
         <is>
-          <t>unlock_wrong</t>
+          <t>data_export_done</t>
         </is>
       </c>
       <c r="C255" s="7" t="inlineStr">
         <is>
-          <t>Buka dengan PIN</t>
+          <t>Datamu</t>
         </is>
       </c>
       <c r="D255" s="7" t="inlineStr">
@@ -9278,15 +9314,19 @@
       </c>
       <c r="E255" s="7" t="inlineStr">
         <is>
-          <t>PIN salah. Coba lagi.</t>
+          <t>Cadangan tersimpan.</t>
         </is>
       </c>
       <c r="F255" s="7" t="inlineStr">
         <is>
-          <t>Wrong PIN. Try again.</t>
-        </is>
-      </c>
-      <c r="G255" s="7" t="inlineStr"/>
+          <t>Backup saved.</t>
+        </is>
+      </c>
+      <c r="G255" s="7" t="inlineStr">
+        <is>
+          <t>Toast after the system save dialog.</t>
+        </is>
+      </c>
       <c r="H255" s="6" t="inlineStr"/>
       <c r="I255" s="6" t="inlineStr"/>
     </row>
@@ -9296,12 +9336,12 @@
       </c>
       <c r="B256" s="7" t="inlineStr">
         <is>
-          <t>unlock_cooldown</t>
+          <t>data_import_cta</t>
         </is>
       </c>
       <c r="C256" s="7" t="inlineStr">
         <is>
-          <t>Buka dengan PIN</t>
+          <t>Datamu</t>
         </is>
       </c>
       <c r="D256" s="7" t="inlineStr">
@@ -9311,159 +9351,151 @@
       </c>
       <c r="E256" s="7" t="inlineStr">
         <is>
-          <t>Terlalu banyak percobaan. Coba lagi dalam {seconds} detik.</t>
+          <t>Pulihkan dari cadangan</t>
         </is>
       </c>
       <c r="F256" s="7" t="inlineStr">
         <is>
-          <t>Too many tries. Try again in {seconds} seconds.</t>
+          <t>Restore from backup</t>
         </is>
       </c>
       <c r="G256" s="7" t="inlineStr">
         <is>
-          <t>After 5 wrong PINs: 30 s cooldown. PLURAL in EN.</t>
+          <t>Without this, the export is useless on a new phone. Proposed for v1.</t>
         </is>
       </c>
       <c r="H256" s="6" t="inlineStr"/>
       <c r="I256" s="6" t="inlineStr"/>
     </row>
     <row r="257">
-      <c r="A257" s="7" t="n">
+      <c r="A257" s="5" t="n">
         <v>256</v>
       </c>
-      <c r="B257" s="7" t="inlineStr">
-        <is>
-          <t>unlock_forgot</t>
-        </is>
-      </c>
-      <c r="C257" s="7" t="inlineStr">
-        <is>
-          <t>Buka dengan PIN</t>
-        </is>
-      </c>
-      <c r="D257" s="7" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="E257" s="7" t="inlineStr">
-        <is>
-          <t>Lupa PIN?</t>
-        </is>
-      </c>
-      <c r="F257" s="7" t="inlineStr">
-        <is>
-          <t>Forgot your PIN?</t>
-        </is>
-      </c>
-      <c r="G257" s="7" t="inlineStr"/>
+      <c r="B257" s="5" t="inlineStr">
+        <is>
+          <t>data_delete_title</t>
+        </is>
+      </c>
+      <c r="C257" s="5" t="inlineStr">
+        <is>
+          <t>Datamu</t>
+        </is>
+      </c>
+      <c r="D257" s="5" t="inlineStr">
+        <is>
+          <t>DESIGN</t>
+        </is>
+      </c>
+      <c r="E257" s="5" t="inlineStr">
+        <is>
+          <t>Hapus semua data</t>
+        </is>
+      </c>
+      <c r="F257" s="5" t="inlineStr">
+        <is>
+          <t>Delete all data</t>
+        </is>
+      </c>
+      <c r="G257" s="5" t="inlineStr"/>
       <c r="H257" s="6" t="inlineStr"/>
       <c r="I257" s="6" t="inlineStr"/>
     </row>
     <row r="258">
-      <c r="A258" s="7" t="n">
+      <c r="A258" s="5" t="n">
         <v>257</v>
       </c>
-      <c r="B258" s="7" t="inlineStr">
-        <is>
-          <t>unlock_forgot_body</t>
-        </is>
-      </c>
-      <c r="C258" s="7" t="inlineStr">
-        <is>
-          <t>Buka dengan PIN</t>
-        </is>
-      </c>
-      <c r="D258" s="7" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="E258" s="7" t="inlineStr">
-        <is>
-          <t>Karena akunmu anonim, PIN tidak bisa dipulihkan. Kamu bisa menghapus data dan mulai dari awal, atau memulihkan dari file cadangan.</t>
-        </is>
-      </c>
-      <c r="F258" s="7" t="inlineStr">
-        <is>
-          <t>Your account is anonymous, so the PIN can't be recovered. You can delete your data and start fresh, or restore from a backup file.</t>
-        </is>
-      </c>
-      <c r="G258" s="7" t="inlineStr">
-        <is>
-          <t>Bottom sheet. Buttons reuse delete_sheet_confirm + data_import_cta + common_cancel.</t>
-        </is>
-      </c>
+      <c r="B258" s="5" t="inlineStr">
+        <is>
+          <t>data_delete_desc</t>
+        </is>
+      </c>
+      <c r="C258" s="5" t="inlineStr">
+        <is>
+          <t>Datamu</t>
+        </is>
+      </c>
+      <c r="D258" s="5" t="inlineStr">
+        <is>
+          <t>DESIGN</t>
+        </is>
+      </c>
+      <c r="E258" s="5" t="inlineStr">
+        <is>
+          <t>Progres, jurnal, dan pengaturan akan hilang permanen.</t>
+        </is>
+      </c>
+      <c r="F258" s="5" t="inlineStr">
+        <is>
+          <t>Your progress, journal and settings will be permanently erased.</t>
+        </is>
+      </c>
+      <c r="G258" s="5" t="inlineStr"/>
       <c r="H258" s="6" t="inlineStr"/>
       <c r="I258" s="6" t="inlineStr"/>
     </row>
     <row r="259">
-      <c r="A259" s="7" t="n">
+      <c r="A259" s="5" t="n">
         <v>258</v>
       </c>
-      <c r="B259" s="7" t="inlineStr">
-        <is>
-          <t>biometric_title</t>
-        </is>
-      </c>
-      <c r="C259" s="7" t="inlineStr">
-        <is>
-          <t>Buka dengan PIN</t>
-        </is>
-      </c>
-      <c r="D259" s="7" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="E259" s="7" t="inlineStr">
-        <is>
-          <t>Buka Izzah</t>
-        </is>
-      </c>
-      <c r="F259" s="7" t="inlineStr">
-        <is>
-          <t>Unlock Izzah</t>
-        </is>
-      </c>
-      <c r="G259" s="7" t="inlineStr">
-        <is>
-          <t>Title of the system BiometricPrompt. Shows the disguise name if a disguise is active.</t>
-        </is>
-      </c>
+      <c r="B259" s="5" t="inlineStr">
+        <is>
+          <t>data_delete_cta</t>
+        </is>
+      </c>
+      <c r="C259" s="5" t="inlineStr">
+        <is>
+          <t>Datamu</t>
+        </is>
+      </c>
+      <c r="D259" s="5" t="inlineStr">
+        <is>
+          <t>DESIGN</t>
+        </is>
+      </c>
+      <c r="E259" s="5" t="inlineStr">
+        <is>
+          <t>Hapus data</t>
+        </is>
+      </c>
+      <c r="F259" s="5" t="inlineStr">
+        <is>
+          <t>Delete data</t>
+        </is>
+      </c>
+      <c r="G259" s="5" t="inlineStr"/>
       <c r="H259" s="6" t="inlineStr"/>
       <c r="I259" s="6" t="inlineStr"/>
     </row>
     <row r="260">
-      <c r="A260" s="7" t="n">
+      <c r="A260" s="5" t="n">
         <v>259</v>
       </c>
-      <c r="B260" s="7" t="inlineStr">
-        <is>
-          <t>biometric_use_pin</t>
-        </is>
-      </c>
-      <c r="C260" s="7" t="inlineStr">
-        <is>
-          <t>Buka dengan PIN</t>
-        </is>
-      </c>
-      <c r="D260" s="7" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="E260" s="7" t="inlineStr">
-        <is>
-          <t>Pakai PIN</t>
-        </is>
-      </c>
-      <c r="F260" s="7" t="inlineStr">
-        <is>
-          <t>Use PIN</t>
-        </is>
-      </c>
-      <c r="G260" s="7" t="inlineStr"/>
+      <c r="B260" s="5" t="inlineStr">
+        <is>
+          <t>delete_sheet_title</t>
+        </is>
+      </c>
+      <c r="C260" s="5" t="inlineStr">
+        <is>
+          <t>Hapus (sheet)</t>
+        </is>
+      </c>
+      <c r="D260" s="5" t="inlineStr">
+        <is>
+          <t>DESIGN</t>
+        </is>
+      </c>
+      <c r="E260" s="5" t="inlineStr">
+        <is>
+          <t>Yakin hapus semua?</t>
+        </is>
+      </c>
+      <c r="F260" s="5" t="inlineStr">
+        <is>
+          <t>Delete everything?</t>
+        </is>
+      </c>
+      <c r="G260" s="5" t="inlineStr"/>
       <c r="H260" s="6" t="inlineStr"/>
       <c r="I260" s="6" t="inlineStr"/>
     </row>
@@ -9473,12 +9505,12 @@
       </c>
       <c r="B261" s="5" t="inlineStr">
         <is>
-          <t>notif_prayer_body</t>
+          <t>delete_sheet_body</t>
         </is>
       </c>
       <c r="C261" s="5" t="inlineStr">
         <is>
-          <t>Notifikasi (sistem)</t>
+          <t>Hapus (sheet)</t>
         </is>
       </c>
       <c r="D261" s="5" t="inlineStr">
@@ -9488,155 +9520,147 @@
       </c>
       <c r="E261" s="5" t="inlineStr">
         <is>
-          <t>Waktunya {prayer}. Sejenak untuk dirimu.</t>
+          <t>Ini tidak bisa dibatalkan. Kalau hanya ingin istirahat, kamu bisa menjeda pengingat saja.</t>
         </is>
       </c>
       <c r="F261" s="5" t="inlineStr">
         <is>
-          <t>Time for {prayer}. A moment for yourself.</t>
-        </is>
-      </c>
-      <c r="G261" s="5" t="inlineStr">
-        <is>
-          <t>RULE: no notification may mention porn, relapse or addiction.</t>
-        </is>
-      </c>
+          <t>This can't be undone. If you just need a break, you can pause the reminders instead.</t>
+        </is>
+      </c>
+      <c r="G261" s="5" t="inlineStr"/>
       <c r="H261" s="6" t="inlineStr"/>
       <c r="I261" s="6" t="inlineStr"/>
     </row>
     <row r="262">
-      <c r="A262" s="7" t="n">
+      <c r="A262" s="5" t="n">
         <v>261</v>
       </c>
-      <c r="B262" s="7" t="inlineStr">
-        <is>
-          <t>notif_dzikir_morning</t>
-        </is>
-      </c>
-      <c r="C262" s="7" t="inlineStr">
-        <is>
-          <t>Notifikasi (sistem)</t>
-        </is>
-      </c>
-      <c r="D262" s="7" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="E262" s="7" t="inlineStr">
-        <is>
-          <t>Pagi yang baru. Ada waktu sebentar untuk dirimu?</t>
-        </is>
-      </c>
-      <c r="F262" s="7" t="inlineStr">
-        <is>
-          <t>A fresh morning. Got a minute for yourself?</t>
-        </is>
-      </c>
-      <c r="G262" s="7" t="inlineStr"/>
+      <c r="B262" s="5" t="inlineStr">
+        <is>
+          <t>delete_sheet_confirm</t>
+        </is>
+      </c>
+      <c r="C262" s="5" t="inlineStr">
+        <is>
+          <t>Hapus (sheet)</t>
+        </is>
+      </c>
+      <c r="D262" s="5" t="inlineStr">
+        <is>
+          <t>DESIGN</t>
+        </is>
+      </c>
+      <c r="E262" s="5" t="inlineStr">
+        <is>
+          <t>Ya, hapus semuanya</t>
+        </is>
+      </c>
+      <c r="F262" s="5" t="inlineStr">
+        <is>
+          <t>Yes, delete everything</t>
+        </is>
+      </c>
+      <c r="G262" s="5" t="inlineStr"/>
       <c r="H262" s="6" t="inlineStr"/>
       <c r="I262" s="6" t="inlineStr"/>
     </row>
     <row r="263">
-      <c r="A263" s="7" t="n">
+      <c r="A263" s="5" t="n">
         <v>262</v>
       </c>
-      <c r="B263" s="7" t="inlineStr">
-        <is>
-          <t>notif_dzikir_evening</t>
-        </is>
-      </c>
-      <c r="C263" s="7" t="inlineStr">
-        <is>
-          <t>Notifikasi (sistem)</t>
-        </is>
-      </c>
-      <c r="D263" s="7" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="E263" s="7" t="inlineStr">
-        <is>
-          <t>Sore menjelang. Sejenak untuk menenangkan hati.</t>
-        </is>
-      </c>
-      <c r="F263" s="7" t="inlineStr">
-        <is>
-          <t>Evening is here. A moment to settle your heart.</t>
-        </is>
-      </c>
-      <c r="G263" s="7" t="inlineStr"/>
+      <c r="B263" s="5" t="inlineStr">
+        <is>
+          <t>common_cancel</t>
+        </is>
+      </c>
+      <c r="C263" s="5" t="inlineStr">
+        <is>
+          <t>Hapus (sheet)</t>
+        </is>
+      </c>
+      <c r="D263" s="5" t="inlineStr">
+        <is>
+          <t>DESIGN</t>
+        </is>
+      </c>
+      <c r="E263" s="5" t="inlineStr">
+        <is>
+          <t>Batal</t>
+        </is>
+      </c>
+      <c r="F263" s="5" t="inlineStr">
+        <is>
+          <t>Cancel</t>
+        </is>
+      </c>
+      <c r="G263" s="5" t="inlineStr"/>
       <c r="H263" s="6" t="inlineStr"/>
       <c r="I263" s="6" t="inlineStr"/>
     </row>
     <row r="264">
-      <c r="A264" s="7" t="n">
+      <c r="A264" s="5" t="n">
         <v>263</v>
       </c>
-      <c r="B264" s="7" t="inlineStr">
-        <is>
-          <t>notif_checkin</t>
-        </is>
-      </c>
-      <c r="C264" s="7" t="inlineStr">
-        <is>
-          <t>Notifikasi (sistem)</t>
-        </is>
-      </c>
-      <c r="D264" s="7" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="E264" s="7" t="inlineStr">
-        <is>
-          <t>Bagaimana harimu? Catat sebentar sebelum istirahat.</t>
-        </is>
-      </c>
-      <c r="F264" s="7" t="inlineStr">
-        <is>
-          <t>How was your day? A quick note before you rest.</t>
-        </is>
-      </c>
-      <c r="G264" s="7" t="inlineStr"/>
+      <c r="B264" s="5" t="inlineStr">
+        <is>
+          <t>unlock_title</t>
+        </is>
+      </c>
+      <c r="C264" s="5" t="inlineStr">
+        <is>
+          <t>Buka dengan PIN</t>
+        </is>
+      </c>
+      <c r="D264" s="5" t="inlineStr">
+        <is>
+          <t>DESIGN</t>
+        </is>
+      </c>
+      <c r="E264" s="5" t="inlineStr">
+        <is>
+          <t>Masukkan PIN</t>
+        </is>
+      </c>
+      <c r="F264" s="5" t="inlineStr">
+        <is>
+          <t>Enter your PIN</t>
+        </is>
+      </c>
+      <c r="G264" s="5" t="inlineStr"/>
       <c r="H264" s="6" t="inlineStr"/>
       <c r="I264" s="6" t="inlineStr"/>
     </row>
     <row r="265">
-      <c r="A265" s="7" t="n">
+      <c r="A265" s="5" t="n">
         <v>264</v>
       </c>
-      <c r="B265" s="7" t="inlineStr">
-        <is>
-          <t>notif_channel_reminders</t>
-        </is>
-      </c>
-      <c r="C265" s="7" t="inlineStr">
-        <is>
-          <t>Notifikasi (sistem)</t>
-        </is>
-      </c>
-      <c r="D265" s="7" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="E265" s="7" t="inlineStr">
-        <is>
-          <t>Pengingat</t>
-        </is>
-      </c>
-      <c r="F265" s="7" t="inlineStr">
-        <is>
-          <t>Reminders</t>
-        </is>
-      </c>
-      <c r="G265" s="7" t="inlineStr">
-        <is>
-          <t>Android notification channel name (visible in system settings).</t>
-        </is>
-      </c>
+      <c r="B265" s="5" t="inlineStr">
+        <is>
+          <t>unlock_subtitle</t>
+        </is>
+      </c>
+      <c r="C265" s="5" t="inlineStr">
+        <is>
+          <t>Buka dengan PIN</t>
+        </is>
+      </c>
+      <c r="D265" s="5" t="inlineStr">
+        <is>
+          <t>DESIGN</t>
+        </is>
+      </c>
+      <c r="E265" s="5" t="inlineStr">
+        <is>
+          <t>Assalamu’alaikum. Selamat datang kembali.</t>
+        </is>
+      </c>
+      <c r="F265" s="5" t="inlineStr">
+        <is>
+          <t>Assalamu’alaikum. Welcome back.</t>
+        </is>
+      </c>
+      <c r="G265" s="5" t="inlineStr"/>
       <c r="H265" s="6" t="inlineStr"/>
       <c r="I265" s="6" t="inlineStr"/>
     </row>
@@ -9646,12 +9670,12 @@
       </c>
       <c r="B266" s="7" t="inlineStr">
         <is>
-          <t>notif_channel_protect</t>
+          <t>unlock_wrong</t>
         </is>
       </c>
       <c r="C266" s="7" t="inlineStr">
         <is>
-          <t>Notifikasi (sistem)</t>
+          <t>Buka dengan PIN</t>
         </is>
       </c>
       <c r="D266" s="7" t="inlineStr">
@@ -9661,19 +9685,15 @@
       </c>
       <c r="E266" s="7" t="inlineStr">
         <is>
-          <t>Penjagaan aktif</t>
+          <t>PIN salah. Coba lagi.</t>
         </is>
       </c>
       <c r="F266" s="7" t="inlineStr">
         <is>
-          <t>Protection running</t>
-        </is>
-      </c>
-      <c r="G266" s="7" t="inlineStr">
-        <is>
-          <t>Foreground service channel for the blocker.</t>
-        </is>
-      </c>
+          <t>Wrong PIN. Try again.</t>
+        </is>
+      </c>
+      <c r="G266" s="7" t="inlineStr"/>
       <c r="H266" s="6" t="inlineStr"/>
       <c r="I266" s="6" t="inlineStr"/>
     </row>
@@ -9683,12 +9703,12 @@
       </c>
       <c r="B267" s="7" t="inlineStr">
         <is>
-          <t>notif_protect_ongoing</t>
+          <t>unlock_cooldown</t>
         </is>
       </c>
       <c r="C267" s="7" t="inlineStr">
         <is>
-          <t>Notifikasi (sistem)</t>
+          <t>Buka dengan PIN</t>
         </is>
       </c>
       <c r="D267" s="7" t="inlineStr">
@@ -9698,155 +9718,159 @@
       </c>
       <c r="E267" s="7" t="inlineStr">
         <is>
-          <t>Berjalan di latar belakang.</t>
+          <t>Terlalu banyak percobaan. Coba lagi dalam {seconds} detik.</t>
         </is>
       </c>
       <c r="F267" s="7" t="inlineStr">
         <is>
-          <t>Running in the background.</t>
+          <t>Too many tries. Try again in {seconds} seconds.</t>
         </is>
       </c>
       <c r="G267" s="7" t="inlineStr">
         <is>
-          <t>Persistent foreground-service notification. Must stay neutral.</t>
+          <t>After 5 wrong PINs: 30 s cooldown. PLURAL in EN.</t>
         </is>
       </c>
       <c r="H267" s="6" t="inlineStr"/>
       <c r="I267" s="6" t="inlineStr"/>
     </row>
     <row r="268">
-      <c r="A268" s="5" t="n">
+      <c r="A268" s="7" t="n">
         <v>267</v>
       </c>
-      <c r="B268" s="5" t="inlineStr">
-        <is>
-          <t>hijri_month_1</t>
-        </is>
-      </c>
-      <c r="C268" s="5" t="inlineStr">
-        <is>
-          <t>Hijri calendar</t>
-        </is>
-      </c>
-      <c r="D268" s="5" t="inlineStr">
-        <is>
-          <t>DESIGN</t>
-        </is>
-      </c>
-      <c r="E268" s="5" t="inlineStr">
-        <is>
-          <t>Muharram</t>
-        </is>
-      </c>
-      <c r="F268" s="5" t="inlineStr">
-        <is>
-          <t>Muharram</t>
-        </is>
-      </c>
-      <c r="G268" s="5" t="inlineStr">
-        <is>
-          <t>Used by {hijri}.</t>
-        </is>
-      </c>
+      <c r="B268" s="7" t="inlineStr">
+        <is>
+          <t>unlock_forgot</t>
+        </is>
+      </c>
+      <c r="C268" s="7" t="inlineStr">
+        <is>
+          <t>Buka dengan PIN</t>
+        </is>
+      </c>
+      <c r="D268" s="7" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="E268" s="7" t="inlineStr">
+        <is>
+          <t>Lupa PIN?</t>
+        </is>
+      </c>
+      <c r="F268" s="7" t="inlineStr">
+        <is>
+          <t>Forgot your PIN?</t>
+        </is>
+      </c>
+      <c r="G268" s="7" t="inlineStr"/>
       <c r="H268" s="6" t="inlineStr"/>
       <c r="I268" s="6" t="inlineStr"/>
     </row>
     <row r="269">
-      <c r="A269" s="5" t="n">
+      <c r="A269" s="7" t="n">
         <v>268</v>
       </c>
-      <c r="B269" s="5" t="inlineStr">
-        <is>
-          <t>hijri_month_2</t>
-        </is>
-      </c>
-      <c r="C269" s="5" t="inlineStr">
-        <is>
-          <t>Hijri calendar</t>
-        </is>
-      </c>
-      <c r="D269" s="5" t="inlineStr">
-        <is>
-          <t>DESIGN</t>
-        </is>
-      </c>
-      <c r="E269" s="5" t="inlineStr">
-        <is>
-          <t>Safar</t>
-        </is>
-      </c>
-      <c r="F269" s="5" t="inlineStr">
-        <is>
-          <t>Safar</t>
-        </is>
-      </c>
-      <c r="G269" s="5" t="inlineStr"/>
+      <c r="B269" s="7" t="inlineStr">
+        <is>
+          <t>unlock_forgot_body</t>
+        </is>
+      </c>
+      <c r="C269" s="7" t="inlineStr">
+        <is>
+          <t>Buka dengan PIN</t>
+        </is>
+      </c>
+      <c r="D269" s="7" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="E269" s="7" t="inlineStr">
+        <is>
+          <t>Karena akunmu anonim, PIN tidak bisa dipulihkan. Kamu bisa menghapus data dan mulai dari awal, atau memulihkan dari file cadangan.</t>
+        </is>
+      </c>
+      <c r="F269" s="7" t="inlineStr">
+        <is>
+          <t>Your account is anonymous, so the PIN can't be recovered. You can delete your data and start fresh, or restore from a backup file.</t>
+        </is>
+      </c>
+      <c r="G269" s="7" t="inlineStr">
+        <is>
+          <t>Bottom sheet. Buttons reuse delete_sheet_confirm + data_import_cta + common_cancel.</t>
+        </is>
+      </c>
       <c r="H269" s="6" t="inlineStr"/>
       <c r="I269" s="6" t="inlineStr"/>
     </row>
     <row r="270">
-      <c r="A270" s="5" t="n">
+      <c r="A270" s="7" t="n">
         <v>269</v>
       </c>
-      <c r="B270" s="5" t="inlineStr">
-        <is>
-          <t>hijri_month_3</t>
-        </is>
-      </c>
-      <c r="C270" s="5" t="inlineStr">
-        <is>
-          <t>Hijri calendar</t>
-        </is>
-      </c>
-      <c r="D270" s="5" t="inlineStr">
-        <is>
-          <t>DESIGN</t>
-        </is>
-      </c>
-      <c r="E270" s="5" t="inlineStr">
-        <is>
-          <t>Rabiul Awal</t>
-        </is>
-      </c>
-      <c r="F270" s="5" t="inlineStr">
-        <is>
-          <t>Rabi‘ al-Awwal</t>
-        </is>
-      </c>
-      <c r="G270" s="5" t="inlineStr"/>
+      <c r="B270" s="7" t="inlineStr">
+        <is>
+          <t>biometric_title</t>
+        </is>
+      </c>
+      <c r="C270" s="7" t="inlineStr">
+        <is>
+          <t>Buka dengan PIN</t>
+        </is>
+      </c>
+      <c r="D270" s="7" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="E270" s="7" t="inlineStr">
+        <is>
+          <t>Buka Izzah</t>
+        </is>
+      </c>
+      <c r="F270" s="7" t="inlineStr">
+        <is>
+          <t>Unlock Izzah</t>
+        </is>
+      </c>
+      <c r="G270" s="7" t="inlineStr">
+        <is>
+          <t>Title of the system BiometricPrompt. Shows the disguise name if a disguise is active.</t>
+        </is>
+      </c>
       <c r="H270" s="6" t="inlineStr"/>
       <c r="I270" s="6" t="inlineStr"/>
     </row>
     <row r="271">
-      <c r="A271" s="5" t="n">
+      <c r="A271" s="7" t="n">
         <v>270</v>
       </c>
-      <c r="B271" s="5" t="inlineStr">
-        <is>
-          <t>hijri_month_4</t>
-        </is>
-      </c>
-      <c r="C271" s="5" t="inlineStr">
-        <is>
-          <t>Hijri calendar</t>
-        </is>
-      </c>
-      <c r="D271" s="5" t="inlineStr">
-        <is>
-          <t>DESIGN</t>
-        </is>
-      </c>
-      <c r="E271" s="5" t="inlineStr">
-        <is>
-          <t>Rabiul Akhir</t>
-        </is>
-      </c>
-      <c r="F271" s="5" t="inlineStr">
-        <is>
-          <t>Rabi‘ al-Thani</t>
-        </is>
-      </c>
-      <c r="G271" s="5" t="inlineStr"/>
+      <c r="B271" s="7" t="inlineStr">
+        <is>
+          <t>biometric_use_pin</t>
+        </is>
+      </c>
+      <c r="C271" s="7" t="inlineStr">
+        <is>
+          <t>Buka dengan PIN</t>
+        </is>
+      </c>
+      <c r="D271" s="7" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="E271" s="7" t="inlineStr">
+        <is>
+          <t>Pakai PIN</t>
+        </is>
+      </c>
+      <c r="F271" s="7" t="inlineStr">
+        <is>
+          <t>Use PIN</t>
+        </is>
+      </c>
+      <c r="G271" s="7" t="inlineStr"/>
       <c r="H271" s="6" t="inlineStr"/>
       <c r="I271" s="6" t="inlineStr"/>
     </row>
@@ -9856,12 +9880,12 @@
       </c>
       <c r="B272" s="5" t="inlineStr">
         <is>
-          <t>hijri_month_5</t>
+          <t>notif_prayer_body</t>
         </is>
       </c>
       <c r="C272" s="5" t="inlineStr">
         <is>
-          <t>Hijri calendar</t>
+          <t>Notifikasi (sistem)</t>
         </is>
       </c>
       <c r="D272" s="5" t="inlineStr">
@@ -9871,213 +9895,229 @@
       </c>
       <c r="E272" s="5" t="inlineStr">
         <is>
-          <t>Jumadil Awal</t>
+          <t>Waktunya {prayer}. Sejenak untuk dirimu.</t>
         </is>
       </c>
       <c r="F272" s="5" t="inlineStr">
         <is>
-          <t>Jumada al-Ula</t>
-        </is>
-      </c>
-      <c r="G272" s="5" t="inlineStr"/>
+          <t>Time for {prayer}. A moment for yourself.</t>
+        </is>
+      </c>
+      <c r="G272" s="5" t="inlineStr">
+        <is>
+          <t>RULE: no notification may mention porn, relapse or addiction.</t>
+        </is>
+      </c>
       <c r="H272" s="6" t="inlineStr"/>
       <c r="I272" s="6" t="inlineStr"/>
     </row>
     <row r="273">
-      <c r="A273" s="5" t="n">
+      <c r="A273" s="7" t="n">
         <v>272</v>
       </c>
-      <c r="B273" s="5" t="inlineStr">
-        <is>
-          <t>hijri_month_6</t>
-        </is>
-      </c>
-      <c r="C273" s="5" t="inlineStr">
-        <is>
-          <t>Hijri calendar</t>
-        </is>
-      </c>
-      <c r="D273" s="5" t="inlineStr">
-        <is>
-          <t>DESIGN</t>
-        </is>
-      </c>
-      <c r="E273" s="5" t="inlineStr">
-        <is>
-          <t>Jumadil Akhir</t>
-        </is>
-      </c>
-      <c r="F273" s="5" t="inlineStr">
-        <is>
-          <t>Jumada al-Akhirah</t>
-        </is>
-      </c>
-      <c r="G273" s="5" t="inlineStr"/>
+      <c r="B273" s="7" t="inlineStr">
+        <is>
+          <t>notif_dzikir_morning</t>
+        </is>
+      </c>
+      <c r="C273" s="7" t="inlineStr">
+        <is>
+          <t>Notifikasi (sistem)</t>
+        </is>
+      </c>
+      <c r="D273" s="7" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="E273" s="7" t="inlineStr">
+        <is>
+          <t>Pagi yang baru. Ada waktu sebentar untuk dirimu?</t>
+        </is>
+      </c>
+      <c r="F273" s="7" t="inlineStr">
+        <is>
+          <t>A fresh morning. Got a minute for yourself?</t>
+        </is>
+      </c>
+      <c r="G273" s="7" t="inlineStr"/>
       <c r="H273" s="6" t="inlineStr"/>
       <c r="I273" s="6" t="inlineStr"/>
     </row>
     <row r="274">
-      <c r="A274" s="5" t="n">
+      <c r="A274" s="7" t="n">
         <v>273</v>
       </c>
-      <c r="B274" s="5" t="inlineStr">
-        <is>
-          <t>hijri_month_7</t>
-        </is>
-      </c>
-      <c r="C274" s="5" t="inlineStr">
-        <is>
-          <t>Hijri calendar</t>
-        </is>
-      </c>
-      <c r="D274" s="5" t="inlineStr">
-        <is>
-          <t>DESIGN</t>
-        </is>
-      </c>
-      <c r="E274" s="5" t="inlineStr">
-        <is>
-          <t>Rajab</t>
-        </is>
-      </c>
-      <c r="F274" s="5" t="inlineStr">
-        <is>
-          <t>Rajab</t>
-        </is>
-      </c>
-      <c r="G274" s="5" t="inlineStr"/>
+      <c r="B274" s="7" t="inlineStr">
+        <is>
+          <t>notif_dzikir_evening</t>
+        </is>
+      </c>
+      <c r="C274" s="7" t="inlineStr">
+        <is>
+          <t>Notifikasi (sistem)</t>
+        </is>
+      </c>
+      <c r="D274" s="7" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="E274" s="7" t="inlineStr">
+        <is>
+          <t>Sore menjelang. Sejenak untuk menenangkan hati.</t>
+        </is>
+      </c>
+      <c r="F274" s="7" t="inlineStr">
+        <is>
+          <t>Evening is here. A moment to settle your heart.</t>
+        </is>
+      </c>
+      <c r="G274" s="7" t="inlineStr"/>
       <c r="H274" s="6" t="inlineStr"/>
       <c r="I274" s="6" t="inlineStr"/>
     </row>
     <row r="275">
-      <c r="A275" s="5" t="n">
+      <c r="A275" s="7" t="n">
         <v>274</v>
       </c>
-      <c r="B275" s="5" t="inlineStr">
-        <is>
-          <t>hijri_month_8</t>
-        </is>
-      </c>
-      <c r="C275" s="5" t="inlineStr">
-        <is>
-          <t>Hijri calendar</t>
-        </is>
-      </c>
-      <c r="D275" s="5" t="inlineStr">
-        <is>
-          <t>DESIGN</t>
-        </is>
-      </c>
-      <c r="E275" s="5" t="inlineStr">
-        <is>
-          <t>Sya’ban</t>
-        </is>
-      </c>
-      <c r="F275" s="5" t="inlineStr">
-        <is>
-          <t>Sha‘ban</t>
-        </is>
-      </c>
-      <c r="G275" s="5" t="inlineStr"/>
+      <c r="B275" s="7" t="inlineStr">
+        <is>
+          <t>notif_checkin</t>
+        </is>
+      </c>
+      <c r="C275" s="7" t="inlineStr">
+        <is>
+          <t>Notifikasi (sistem)</t>
+        </is>
+      </c>
+      <c r="D275" s="7" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="E275" s="7" t="inlineStr">
+        <is>
+          <t>Bagaimana harimu? Catat sebentar sebelum istirahat.</t>
+        </is>
+      </c>
+      <c r="F275" s="7" t="inlineStr">
+        <is>
+          <t>How was your day? A quick note before you rest.</t>
+        </is>
+      </c>
+      <c r="G275" s="7" t="inlineStr"/>
       <c r="H275" s="6" t="inlineStr"/>
       <c r="I275" s="6" t="inlineStr"/>
     </row>
     <row r="276">
-      <c r="A276" s="5" t="n">
+      <c r="A276" s="7" t="n">
         <v>275</v>
       </c>
-      <c r="B276" s="5" t="inlineStr">
-        <is>
-          <t>hijri_month_9</t>
-        </is>
-      </c>
-      <c r="C276" s="5" t="inlineStr">
-        <is>
-          <t>Hijri calendar</t>
-        </is>
-      </c>
-      <c r="D276" s="5" t="inlineStr">
-        <is>
-          <t>DESIGN</t>
-        </is>
-      </c>
-      <c r="E276" s="5" t="inlineStr">
-        <is>
-          <t>Ramadhan</t>
-        </is>
-      </c>
-      <c r="F276" s="5" t="inlineStr">
-        <is>
-          <t>Ramadan</t>
-        </is>
-      </c>
-      <c r="G276" s="5" t="inlineStr"/>
+      <c r="B276" s="7" t="inlineStr">
+        <is>
+          <t>notif_channel_reminders</t>
+        </is>
+      </c>
+      <c r="C276" s="7" t="inlineStr">
+        <is>
+          <t>Notifikasi (sistem)</t>
+        </is>
+      </c>
+      <c r="D276" s="7" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="E276" s="7" t="inlineStr">
+        <is>
+          <t>Pengingat</t>
+        </is>
+      </c>
+      <c r="F276" s="7" t="inlineStr">
+        <is>
+          <t>Reminders</t>
+        </is>
+      </c>
+      <c r="G276" s="7" t="inlineStr">
+        <is>
+          <t>Android notification channel name (visible in system settings).</t>
+        </is>
+      </c>
       <c r="H276" s="6" t="inlineStr"/>
       <c r="I276" s="6" t="inlineStr"/>
     </row>
     <row r="277">
-      <c r="A277" s="5" t="n">
+      <c r="A277" s="7" t="n">
         <v>276</v>
       </c>
-      <c r="B277" s="5" t="inlineStr">
-        <is>
-          <t>hijri_month_10</t>
-        </is>
-      </c>
-      <c r="C277" s="5" t="inlineStr">
-        <is>
-          <t>Hijri calendar</t>
-        </is>
-      </c>
-      <c r="D277" s="5" t="inlineStr">
-        <is>
-          <t>DESIGN</t>
-        </is>
-      </c>
-      <c r="E277" s="5" t="inlineStr">
-        <is>
-          <t>Syawal</t>
-        </is>
-      </c>
-      <c r="F277" s="5" t="inlineStr">
-        <is>
-          <t>Shawwal</t>
-        </is>
-      </c>
-      <c r="G277" s="5" t="inlineStr"/>
+      <c r="B277" s="7" t="inlineStr">
+        <is>
+          <t>notif_channel_protect</t>
+        </is>
+      </c>
+      <c r="C277" s="7" t="inlineStr">
+        <is>
+          <t>Notifikasi (sistem)</t>
+        </is>
+      </c>
+      <c r="D277" s="7" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="E277" s="7" t="inlineStr">
+        <is>
+          <t>Penjagaan aktif</t>
+        </is>
+      </c>
+      <c r="F277" s="7" t="inlineStr">
+        <is>
+          <t>Protection running</t>
+        </is>
+      </c>
+      <c r="G277" s="7" t="inlineStr">
+        <is>
+          <t>Foreground service channel for the blocker.</t>
+        </is>
+      </c>
       <c r="H277" s="6" t="inlineStr"/>
       <c r="I277" s="6" t="inlineStr"/>
     </row>
     <row r="278">
-      <c r="A278" s="5" t="n">
+      <c r="A278" s="7" t="n">
         <v>277</v>
       </c>
-      <c r="B278" s="5" t="inlineStr">
-        <is>
-          <t>hijri_month_11</t>
-        </is>
-      </c>
-      <c r="C278" s="5" t="inlineStr">
-        <is>
-          <t>Hijri calendar</t>
-        </is>
-      </c>
-      <c r="D278" s="5" t="inlineStr">
-        <is>
-          <t>DESIGN</t>
-        </is>
-      </c>
-      <c r="E278" s="5" t="inlineStr">
-        <is>
-          <t>Dzulqa’dah</t>
-        </is>
-      </c>
-      <c r="F278" s="5" t="inlineStr">
-        <is>
-          <t>Dhu al-Qa‘dah</t>
-        </is>
-      </c>
-      <c r="G278" s="5" t="inlineStr"/>
+      <c r="B278" s="7" t="inlineStr">
+        <is>
+          <t>notif_protect_ongoing</t>
+        </is>
+      </c>
+      <c r="C278" s="7" t="inlineStr">
+        <is>
+          <t>Notifikasi (sistem)</t>
+        </is>
+      </c>
+      <c r="D278" s="7" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="E278" s="7" t="inlineStr">
+        <is>
+          <t>Berjalan di latar belakang.</t>
+        </is>
+      </c>
+      <c r="F278" s="7" t="inlineStr">
+        <is>
+          <t>Running in the background.</t>
+        </is>
+      </c>
+      <c r="G278" s="7" t="inlineStr">
+        <is>
+          <t>Persistent foreground-service notification. Must stay neutral.</t>
+        </is>
+      </c>
       <c r="H278" s="6" t="inlineStr"/>
       <c r="I278" s="6" t="inlineStr"/>
     </row>
@@ -10087,7 +10127,7 @@
       </c>
       <c r="B279" s="5" t="inlineStr">
         <is>
-          <t>hijri_month_12</t>
+          <t>hijri_month_1</t>
         </is>
       </c>
       <c r="C279" s="5" t="inlineStr">
@@ -10102,15 +10142,19 @@
       </c>
       <c r="E279" s="5" t="inlineStr">
         <is>
-          <t>Dzulhijjah</t>
+          <t>Muharram</t>
         </is>
       </c>
       <c r="F279" s="5" t="inlineStr">
         <is>
-          <t>Dhu al-Hijjah</t>
-        </is>
-      </c>
-      <c r="G279" s="5" t="inlineStr"/>
+          <t>Muharram</t>
+        </is>
+      </c>
+      <c r="G279" s="5" t="inlineStr">
+        <is>
+          <t>Used by {hijri}.</t>
+        </is>
+      </c>
       <c r="H279" s="6" t="inlineStr"/>
       <c r="I279" s="6" t="inlineStr"/>
     </row>
@@ -10120,7 +10164,7 @@
       </c>
       <c r="B280" s="5" t="inlineStr">
         <is>
-          <t>hijri_suffix</t>
+          <t>hijri_month_2</t>
         </is>
       </c>
       <c r="C280" s="5" t="inlineStr">
@@ -10135,22 +10179,385 @@
       </c>
       <c r="E280" s="5" t="inlineStr">
         <is>
-          <t>{day} {month} {year} H</t>
+          <t>Safar</t>
         </is>
       </c>
       <c r="F280" s="5" t="inlineStr">
         <is>
-          <t>{day} {month} {year} AH</t>
+          <t>Safar</t>
         </is>
       </c>
       <c r="G280" s="5" t="inlineStr"/>
       <c r="H280" s="6" t="inlineStr"/>
       <c r="I280" s="6" t="inlineStr"/>
     </row>
+    <row r="281">
+      <c r="A281" s="5" t="n">
+        <v>280</v>
+      </c>
+      <c r="B281" s="5" t="inlineStr">
+        <is>
+          <t>hijri_month_3</t>
+        </is>
+      </c>
+      <c r="C281" s="5" t="inlineStr">
+        <is>
+          <t>Hijri calendar</t>
+        </is>
+      </c>
+      <c r="D281" s="5" t="inlineStr">
+        <is>
+          <t>DESIGN</t>
+        </is>
+      </c>
+      <c r="E281" s="5" t="inlineStr">
+        <is>
+          <t>Rabiul Awal</t>
+        </is>
+      </c>
+      <c r="F281" s="5" t="inlineStr">
+        <is>
+          <t>Rabi‘ al-Awwal</t>
+        </is>
+      </c>
+      <c r="G281" s="5" t="inlineStr"/>
+      <c r="H281" s="6" t="inlineStr"/>
+      <c r="I281" s="6" t="inlineStr"/>
+    </row>
+    <row r="282">
+      <c r="A282" s="5" t="n">
+        <v>281</v>
+      </c>
+      <c r="B282" s="5" t="inlineStr">
+        <is>
+          <t>hijri_month_4</t>
+        </is>
+      </c>
+      <c r="C282" s="5" t="inlineStr">
+        <is>
+          <t>Hijri calendar</t>
+        </is>
+      </c>
+      <c r="D282" s="5" t="inlineStr">
+        <is>
+          <t>DESIGN</t>
+        </is>
+      </c>
+      <c r="E282" s="5" t="inlineStr">
+        <is>
+          <t>Rabiul Akhir</t>
+        </is>
+      </c>
+      <c r="F282" s="5" t="inlineStr">
+        <is>
+          <t>Rabi‘ al-Thani</t>
+        </is>
+      </c>
+      <c r="G282" s="5" t="inlineStr"/>
+      <c r="H282" s="6" t="inlineStr"/>
+      <c r="I282" s="6" t="inlineStr"/>
+    </row>
+    <row r="283">
+      <c r="A283" s="5" t="n">
+        <v>282</v>
+      </c>
+      <c r="B283" s="5" t="inlineStr">
+        <is>
+          <t>hijri_month_5</t>
+        </is>
+      </c>
+      <c r="C283" s="5" t="inlineStr">
+        <is>
+          <t>Hijri calendar</t>
+        </is>
+      </c>
+      <c r="D283" s="5" t="inlineStr">
+        <is>
+          <t>DESIGN</t>
+        </is>
+      </c>
+      <c r="E283" s="5" t="inlineStr">
+        <is>
+          <t>Jumadil Awal</t>
+        </is>
+      </c>
+      <c r="F283" s="5" t="inlineStr">
+        <is>
+          <t>Jumada al-Ula</t>
+        </is>
+      </c>
+      <c r="G283" s="5" t="inlineStr"/>
+      <c r="H283" s="6" t="inlineStr"/>
+      <c r="I283" s="6" t="inlineStr"/>
+    </row>
+    <row r="284">
+      <c r="A284" s="5" t="n">
+        <v>283</v>
+      </c>
+      <c r="B284" s="5" t="inlineStr">
+        <is>
+          <t>hijri_month_6</t>
+        </is>
+      </c>
+      <c r="C284" s="5" t="inlineStr">
+        <is>
+          <t>Hijri calendar</t>
+        </is>
+      </c>
+      <c r="D284" s="5" t="inlineStr">
+        <is>
+          <t>DESIGN</t>
+        </is>
+      </c>
+      <c r="E284" s="5" t="inlineStr">
+        <is>
+          <t>Jumadil Akhir</t>
+        </is>
+      </c>
+      <c r="F284" s="5" t="inlineStr">
+        <is>
+          <t>Jumada al-Akhirah</t>
+        </is>
+      </c>
+      <c r="G284" s="5" t="inlineStr"/>
+      <c r="H284" s="6" t="inlineStr"/>
+      <c r="I284" s="6" t="inlineStr"/>
+    </row>
+    <row r="285">
+      <c r="A285" s="5" t="n">
+        <v>284</v>
+      </c>
+      <c r="B285" s="5" t="inlineStr">
+        <is>
+          <t>hijri_month_7</t>
+        </is>
+      </c>
+      <c r="C285" s="5" t="inlineStr">
+        <is>
+          <t>Hijri calendar</t>
+        </is>
+      </c>
+      <c r="D285" s="5" t="inlineStr">
+        <is>
+          <t>DESIGN</t>
+        </is>
+      </c>
+      <c r="E285" s="5" t="inlineStr">
+        <is>
+          <t>Rajab</t>
+        </is>
+      </c>
+      <c r="F285" s="5" t="inlineStr">
+        <is>
+          <t>Rajab</t>
+        </is>
+      </c>
+      <c r="G285" s="5" t="inlineStr"/>
+      <c r="H285" s="6" t="inlineStr"/>
+      <c r="I285" s="6" t="inlineStr"/>
+    </row>
+    <row r="286">
+      <c r="A286" s="5" t="n">
+        <v>285</v>
+      </c>
+      <c r="B286" s="5" t="inlineStr">
+        <is>
+          <t>hijri_month_8</t>
+        </is>
+      </c>
+      <c r="C286" s="5" t="inlineStr">
+        <is>
+          <t>Hijri calendar</t>
+        </is>
+      </c>
+      <c r="D286" s="5" t="inlineStr">
+        <is>
+          <t>DESIGN</t>
+        </is>
+      </c>
+      <c r="E286" s="5" t="inlineStr">
+        <is>
+          <t>Sya’ban</t>
+        </is>
+      </c>
+      <c r="F286" s="5" t="inlineStr">
+        <is>
+          <t>Sha‘ban</t>
+        </is>
+      </c>
+      <c r="G286" s="5" t="inlineStr"/>
+      <c r="H286" s="6" t="inlineStr"/>
+      <c r="I286" s="6" t="inlineStr"/>
+    </row>
+    <row r="287">
+      <c r="A287" s="5" t="n">
+        <v>286</v>
+      </c>
+      <c r="B287" s="5" t="inlineStr">
+        <is>
+          <t>hijri_month_9</t>
+        </is>
+      </c>
+      <c r="C287" s="5" t="inlineStr">
+        <is>
+          <t>Hijri calendar</t>
+        </is>
+      </c>
+      <c r="D287" s="5" t="inlineStr">
+        <is>
+          <t>DESIGN</t>
+        </is>
+      </c>
+      <c r="E287" s="5" t="inlineStr">
+        <is>
+          <t>Ramadhan</t>
+        </is>
+      </c>
+      <c r="F287" s="5" t="inlineStr">
+        <is>
+          <t>Ramadan</t>
+        </is>
+      </c>
+      <c r="G287" s="5" t="inlineStr"/>
+      <c r="H287" s="6" t="inlineStr"/>
+      <c r="I287" s="6" t="inlineStr"/>
+    </row>
+    <row r="288">
+      <c r="A288" s="5" t="n">
+        <v>287</v>
+      </c>
+      <c r="B288" s="5" t="inlineStr">
+        <is>
+          <t>hijri_month_10</t>
+        </is>
+      </c>
+      <c r="C288" s="5" t="inlineStr">
+        <is>
+          <t>Hijri calendar</t>
+        </is>
+      </c>
+      <c r="D288" s="5" t="inlineStr">
+        <is>
+          <t>DESIGN</t>
+        </is>
+      </c>
+      <c r="E288" s="5" t="inlineStr">
+        <is>
+          <t>Syawal</t>
+        </is>
+      </c>
+      <c r="F288" s="5" t="inlineStr">
+        <is>
+          <t>Shawwal</t>
+        </is>
+      </c>
+      <c r="G288" s="5" t="inlineStr"/>
+      <c r="H288" s="6" t="inlineStr"/>
+      <c r="I288" s="6" t="inlineStr"/>
+    </row>
+    <row r="289">
+      <c r="A289" s="5" t="n">
+        <v>288</v>
+      </c>
+      <c r="B289" s="5" t="inlineStr">
+        <is>
+          <t>hijri_month_11</t>
+        </is>
+      </c>
+      <c r="C289" s="5" t="inlineStr">
+        <is>
+          <t>Hijri calendar</t>
+        </is>
+      </c>
+      <c r="D289" s="5" t="inlineStr">
+        <is>
+          <t>DESIGN</t>
+        </is>
+      </c>
+      <c r="E289" s="5" t="inlineStr">
+        <is>
+          <t>Dzulqa’dah</t>
+        </is>
+      </c>
+      <c r="F289" s="5" t="inlineStr">
+        <is>
+          <t>Dhu al-Qa‘dah</t>
+        </is>
+      </c>
+      <c r="G289" s="5" t="inlineStr"/>
+      <c r="H289" s="6" t="inlineStr"/>
+      <c r="I289" s="6" t="inlineStr"/>
+    </row>
+    <row r="290">
+      <c r="A290" s="5" t="n">
+        <v>289</v>
+      </c>
+      <c r="B290" s="5" t="inlineStr">
+        <is>
+          <t>hijri_month_12</t>
+        </is>
+      </c>
+      <c r="C290" s="5" t="inlineStr">
+        <is>
+          <t>Hijri calendar</t>
+        </is>
+      </c>
+      <c r="D290" s="5" t="inlineStr">
+        <is>
+          <t>DESIGN</t>
+        </is>
+      </c>
+      <c r="E290" s="5" t="inlineStr">
+        <is>
+          <t>Dzulhijjah</t>
+        </is>
+      </c>
+      <c r="F290" s="5" t="inlineStr">
+        <is>
+          <t>Dhu al-Hijjah</t>
+        </is>
+      </c>
+      <c r="G290" s="5" t="inlineStr"/>
+      <c r="H290" s="6" t="inlineStr"/>
+      <c r="I290" s="6" t="inlineStr"/>
+    </row>
+    <row r="291">
+      <c r="A291" s="5" t="n">
+        <v>290</v>
+      </c>
+      <c r="B291" s="5" t="inlineStr">
+        <is>
+          <t>hijri_suffix</t>
+        </is>
+      </c>
+      <c r="C291" s="5" t="inlineStr">
+        <is>
+          <t>Hijri calendar</t>
+        </is>
+      </c>
+      <c r="D291" s="5" t="inlineStr">
+        <is>
+          <t>DESIGN</t>
+        </is>
+      </c>
+      <c r="E291" s="5" t="inlineStr">
+        <is>
+          <t>{day} {month} {year} H</t>
+        </is>
+      </c>
+      <c r="F291" s="5" t="inlineStr">
+        <is>
+          <t>{day} {month} {year} AH</t>
+        </is>
+      </c>
+      <c r="G291" s="5" t="inlineStr"/>
+      <c r="H291" s="6" t="inlineStr"/>
+      <c r="I291" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I280"/>
+  <autoFilter ref="A1:I291"/>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H280" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H2:H291" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"OK,Revisi,Hapus"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>